<commit_message>
Reforça fidelidade de espessura de correntes nos prompts (v3)
Peças com corrente estavam saindo com elos/fios visivelmente mais
grossos do que a peça real — erro clássico de geração por IA (correntes
finas são ambíguas visualmente e o modelo tende a "engordar" pra algo
mais parecido com o que viu mais no treinamento). Adiciona instrução
explícita no bloco de fidelidade, aplicada aos 134 prompts: a espessura
e o diâmetro do elo devem ser idênticos ao original, nunca mais
grossos/vistosos, mesmo que fique mais sutil na imagem gerada.
</commit_message>
<xml_diff>
--- a/content/Photo_Studio_TPV_Biblioteca_de_Prompts.xlsx
+++ b/content/Photo_Studio_TPV_Biblioteca_de_Prompts.xlsx
@@ -721,7 +721,7 @@
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -771,7 +771,7 @@
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto) — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -817,7 +817,7 @@
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -863,7 +863,7 @@
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -913,7 +913,7 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto) usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -959,7 +959,7 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -1055,7 +1055,7 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a peça em uma curva aberta e levemente assimétrica sobre a superfície, sugerindo o formato do pescoço sem formar um círculo perfeito ou fechado.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -1247,7 +1247,7 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pescoço, evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pescoço — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -1293,7 +1293,7 @@
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a peça em uma curva aberta e levemente assimétrica sobre a superfície, sugerindo o formato do pescoço sem formar um círculo perfeito ou fechado.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -1339,7 +1339,7 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a peça em uma curva aberta e levemente assimétrica sobre a superfície, sugerindo o formato do pescoço sem formar um círculo perfeito ou fechado.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pescoço, evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em o pescoço usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -1435,7 +1435,7 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a corrente formando curvas amplas, orgânicas e assimétricas — nunca curvas espelhadas ou geométricas. Deixe o pingente (ou uma das extremidades) como ponto focal da composição, com o restante se estendendo de forma natural, como se tivesse acabado de cair sobre a superfície.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -1485,7 +1485,7 @@
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo e o decote, evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo e o decote — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -1531,7 +1531,7 @@
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a corrente formando curvas amplas, orgânicas e assimétricas — nunca curvas espelhadas ou geométricas. Deixe o pingente (ou uma das extremidades) como ponto focal da composição, com o restante se estendendo de forma natural, como se tivesse acabado de cair sobre a superfície.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -1577,7 +1577,7 @@
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a corrente formando curvas amplas, orgânicas e assimétricas — nunca curvas espelhadas ou geométricas. Deixe o pingente (ou uma das extremidades) como ponto focal da composição, com o restante se estendendo de forma natural, como se tivesse acabado de cair sobre a superfície.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -1627,7 +1627,7 @@
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo e o decote, evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em o colo e o decote usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o pingente como protagonista absoluto, com a corrente caindo ao redor em curvas orgânicas e assimétricas — nunca círculos, ovais ou formas espelhadas dos dois lados.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -1723,7 +1723,7 @@
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo, próximo ao centro do peito, evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, próximo ao centro do peito — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -1769,7 +1769,7 @@
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o pingente como protagonista absoluto, com a corrente caindo ao redor em curvas orgânicas e assimétricas — nunca círculos, ovais ou formas espelhadas dos dois lados.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -1815,7 +1815,7 @@
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o pingente como protagonista absoluto, com a corrente caindo ao redor em curvas orgânicas e assimétricas — nunca círculos, ovais ou formas espelhadas dos dois lados.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -1865,7 +1865,7 @@
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo, próximo ao centro do peito, evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em o colo, próximo ao centro do peito usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -1911,7 +1911,7 @@
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a corrente em uma curva reta a levemente ondulada, transmitindo peso e robustez — nunca curvas perfeitamente simétricas ou decorativas demais.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -1961,7 +1961,7 @@
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o peito e a base do pescoço, com estilo masculino, evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o peito e a base do pescoço, com estilo masculino — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -2007,7 +2007,7 @@
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a corrente em uma curva reta a levemente ondulada, transmitindo peso e robustez — nunca curvas perfeitamente simétricas ou decorativas demais.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -2053,7 +2053,7 @@
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a corrente em uma curva reta a levemente ondulada, transmitindo peso e robustez — nunca curvas perfeitamente simétricas ou decorativas demais.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o peito e a base do pescoço, com estilo masculino, evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em o peito e a base do pescoço, com estilo masculino usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -2149,7 +2149,7 @@
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -2199,7 +2199,7 @@
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -2245,7 +2245,7 @@
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -2291,7 +2291,7 @@
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -2341,7 +2341,7 @@
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em o pulso usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -2387,7 +2387,7 @@
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o bracelete em pé, com o eixo central perpendicular à superfície (aproximadamente 90°) e inclinação máxima de 3° — o suficiente apenas para evitar aparência artificial de renderização. O centro de gravidade deve estar exatamente sobre o ponto de apoio, sem parecer tombado ou flutuando. A peça deve ocupar cerca de 65% da altura da imagem.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -2437,7 +2437,7 @@
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso e o antebraço, evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso e o antebraço — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o bracelete em pé, com o eixo central perpendicular à superfície (aproximadamente 90°) e inclinação máxima de 3° — o suficiente apenas para evitar aparência artificial de renderização. O centro de gravidade deve estar exatamente sobre o ponto de apoio, sem parecer tombado ou flutuando. A peça deve ocupar cerca de 65% da altura da imagem.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -2529,7 +2529,7 @@
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o bracelete em pé, com o eixo central perpendicular à superfície (aproximadamente 90°) e inclinação máxima de 3° — o suficiente apenas para evitar aparência artificial de renderização. O centro de gravidade deve estar exatamente sobre o ponto de apoio, sem parecer tombado ou flutuando. A peça deve ocupar cerca de 65% da altura da imagem.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -2579,7 +2579,7 @@
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso e o antebraço, evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em o pulso e o antebraço usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -2625,7 +2625,7 @@
       </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -2675,7 +2675,7 @@
       </c>
       <c r="G43" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a mão e os dedos — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -2721,7 +2721,7 @@
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -2767,7 +2767,7 @@
       </c>
       <c r="G45" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -2817,7 +2817,7 @@
       </c>
       <c r="G46" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em a mão e os dedos usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -2863,7 +2863,7 @@
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione as duas alianças em pé, lado a lado, uma levemente sobreposta à outra, ambas fisicamente equilibradas sobre a superfície — nunca flutuando.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -2913,7 +2913,7 @@
       </c>
       <c r="G48" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas as mãos entrelaçadas, próximas ao dedo anelar, evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas as mãos entrelaçadas, próximas ao dedo anelar — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -2959,7 +2959,7 @@
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione as duas alianças em pé, lado a lado, uma levemente sobreposta à outra, ambas fisicamente equilibradas sobre a superfície — nunca flutuando.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -3005,7 +3005,7 @@
       </c>
       <c r="G50" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione as duas alianças em pé, lado a lado, uma levemente sobreposta à outra, ambas fisicamente equilibradas sobre a superfície — nunca flutuando.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -3055,7 +3055,7 @@
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas as mãos entrelaçadas, próximas ao dedo anelar, evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em as mãos entrelaçadas, próximas ao dedo anelar usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -3101,7 +3101,7 @@
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a peça formando uma curva aberta e natural, como se tivesse caído sobre a superfície — nunca um círculo perfeitamente fechado.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -3151,7 +3151,7 @@
       </c>
       <c r="G53" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o tornozelo e o pé, evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o tornozelo e o pé — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -3197,7 +3197,7 @@
       </c>
       <c r="G54" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a peça formando uma curva aberta e natural, como se tivesse caído sobre a superfície — nunca um círculo perfeitamente fechado.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -3243,7 +3243,7 @@
       </c>
       <c r="G55" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a peça formando uma curva aberta e natural, como se tivesse caído sobre a superfície — nunca um círculo perfeitamente fechado.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -3293,7 +3293,7 @@
       </c>
       <c r="G56" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o tornozelo e o pé, evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em o tornozelo e o pé usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -3339,7 +3339,7 @@
       </c>
       <c r="G57" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o broche sobre uma prega de tecido, mostrando claramente o pino e o relevo frontal da peça, sem parecer flutuando.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -3389,7 +3389,7 @@
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a lapela de um blazer ou prega de tecido, evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a lapela de um blazer ou prega de tecido — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -3435,7 +3435,7 @@
       </c>
       <c r="G59" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o broche sobre uma prega de tecido, mostrando claramente o pino e o relevo frontal da peça, sem parecer flutuando.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -3481,7 +3481,7 @@
       </c>
       <c r="G60" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o broche sobre uma prega de tecido, mostrando claramente o pino e o relevo frontal da peça, sem parecer flutuando.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="G61" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a lapela de um blazer ou prega de tecido, evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em a lapela de um blazer ou prega de tecido usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -3577,7 +3577,7 @@
       </c>
       <c r="G62" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Utilize exatamente as peças presentes na foto anexada, na mesma quantidade — nunca adicione, remova ou duplique nenhuma joia. Se não houver um tipo de peça na foto, não crie esse tipo de peça. Organize cada peça de acordo com seu próprio comportamento físico (colar em curvas orgânicas e assimétricas; brincos próximos entre si, mostrando a face principal), distribuindo os elementos em diferentes regiões da composição para um equilíbrio visual sofisticado, porém não perfeitamente simétrico.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -3627,7 +3627,7 @@
       </c>
       <c r="G63" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pescoço, o colo e a orelha, evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pescoço, o colo e a orelha — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -3673,7 +3673,7 @@
       </c>
       <c r="G64" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Utilize exatamente as peças presentes na foto anexada, na mesma quantidade — nunca adicione, remova ou duplique nenhuma joia. Se não houver um tipo de peça na foto, não crie esse tipo de peça. Organize cada peça de acordo com seu próprio comportamento físico (colar em curvas orgânicas e assimétricas; brincos próximos entre si, mostrando a face principal), distribuindo os elementos em diferentes regiões da composição para um equilíbrio visual sofisticado, porém não perfeitamente simétrico.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -3719,7 +3719,7 @@
       </c>
       <c r="G65" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Utilize exatamente as peças presentes na foto anexada, na mesma quantidade — nunca adicione, remova ou duplique nenhuma joia. Se não houver um tipo de peça na foto, não crie esse tipo de peça. Organize cada peça de acordo com seu próprio comportamento físico (colar em curvas orgânicas e assimétricas; brincos próximos entre si, mostrando a face principal), distribuindo os elementos em diferentes regiões da composição para um equilíbrio visual sofisticado, porém não perfeitamente simétrico.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -3769,7 +3769,7 @@
       </c>
       <c r="G66" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pescoço, o colo e a orelha, evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em o pescoço, o colo e a orelha usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -3815,7 +3815,7 @@
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o relógio em pé, mostrando o mostrador de frente, com a pulseira formando uma curva aberta e natural ao redor — fisicamente equilibrado, nunca flutuando ou tombado.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -3865,7 +3865,7 @@
       </c>
       <c r="G68" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -3911,7 +3911,7 @@
       </c>
       <c r="G69" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o relógio em pé, mostrando o mostrador de frente, com a pulseira formando uma curva aberta e natural ao redor — fisicamente equilibrado, nunca flutuando ou tombado.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -3957,7 +3957,7 @@
       </c>
       <c r="G70" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o relógio em pé, mostrando o mostrador de frente, com a pulseira formando uma curva aberta e natural ao redor — fisicamente equilibrado, nunca flutuando ou tombado.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -4007,7 +4007,7 @@
       </c>
       <c r="G71" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em o pulso usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
@@ -4149,7 +4149,7 @@
       </c>
       <c r="H2" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
 Tema visual: Dia das Mães. Paleta de cores: tons de rosa suave e nude. Elementos/props de cena: flores (rosas) desfocadas ao fundo, tecido de seda rosa-claro. Clima geral: afetivo, delicado e caloroso.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -4205,7 +4205,7 @@
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
 Tema visual: Dia das Mães. Paleta de cores: tons de rosa suave e nude. Elementos/props de cena: flores (rosas) desfocadas ao fundo, tecido de seda rosa-claro. Clima geral: afetivo, delicado e caloroso.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto) — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -4257,7 +4257,7 @@
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
 Tema visual: Dia das Mães. Paleta de cores: tons de rosa suave e nude. Elementos/props de cena: flores (rosas) desfocadas ao fundo, tecido de seda rosa-claro. Clima geral: afetivo, delicado e caloroso.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -4313,7 +4313,7 @@
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
 Tema visual: Dia das Mães. Paleta de cores: tons de rosa suave e nude. Elementos/props de cena: flores (rosas) desfocadas ao fundo, tecido de seda rosa-claro. Clima geral: afetivo, delicado e caloroso.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -4365,7 +4365,7 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
 Tema visual: Dia das Mães. Paleta de cores: tons de rosa suave e nude. Elementos/props de cena: flores (rosas) desfocadas ao fundo, tecido de seda rosa-claro. Clima geral: afetivo, delicado e caloroso.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -4421,7 +4421,7 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
 Tema visual: Dia das Mães. Paleta de cores: tons de rosa suave e nude. Elementos/props de cena: flores (rosas) desfocadas ao fundo, tecido de seda rosa-claro. Clima geral: afetivo, delicado e caloroso.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a mão e os dedos — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -4473,7 +4473,7 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
 Tema visual: Dia das Mães. Paleta de cores: tons de rosa suave e nude. Elementos/props de cena: flores (rosas) desfocadas ao fundo, tecido de seda rosa-claro. Clima geral: afetivo, delicado e caloroso.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -4529,7 +4529,7 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
 Tema visual: Dia das Mães. Paleta de cores: tons de rosa suave e nude. Elementos/props de cena: flores (rosas) desfocadas ao fundo, tecido de seda rosa-claro. Clima geral: afetivo, delicado e caloroso.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -4581,7 +4581,7 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
 Tema visual: Dia dos Namorados. Paleta de cores: tons de vermelho e vinho. Elementos/props de cena: pétalas de rosa vermelha, velas acesas desfocadas ao fundo. Clima geral: romântico, intimista, iluminação quente e noturna.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -4637,7 +4637,7 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
 Tema visual: Dia dos Namorados. Paleta de cores: tons de vermelho e vinho. Elementos/props de cena: pétalas de rosa vermelha, velas acesas desfocadas ao fundo. Clima geral: romântico, intimista, iluminação quente e noturna.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto) — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -4689,7 +4689,7 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
 Tema visual: Dia dos Namorados. Paleta de cores: tons de vermelho e vinho. Elementos/props de cena: pétalas de rosa vermelha, velas acesas desfocadas ao fundo. Clima geral: romântico, intimista, iluminação quente e noturna.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -4745,7 +4745,7 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
 Tema visual: Dia dos Namorados. Paleta de cores: tons de vermelho e vinho. Elementos/props de cena: pétalas de rosa vermelha, velas acesas desfocadas ao fundo. Clima geral: romântico, intimista, iluminação quente e noturna.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -4797,7 +4797,7 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
 Tema visual: Dia dos Namorados. Paleta de cores: tons de vermelho e vinho. Elementos/props de cena: pétalas de rosa vermelha, velas acesas desfocadas ao fundo. Clima geral: romântico, intimista, iluminação quente e noturna.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -4853,7 +4853,7 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
 Tema visual: Dia dos Namorados. Paleta de cores: tons de vermelho e vinho. Elementos/props de cena: pétalas de rosa vermelha, velas acesas desfocadas ao fundo. Clima geral: romântico, intimista, iluminação quente e noturna.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a mão e os dedos — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -4905,7 +4905,7 @@
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
 Tema visual: Dia dos Namorados. Paleta de cores: tons de vermelho e vinho. Elementos/props de cena: pétalas de rosa vermelha, velas acesas desfocadas ao fundo. Clima geral: romântico, intimista, iluminação quente e noturna.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -4961,7 +4961,7 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
 Tema visual: Dia dos Namorados. Paleta de cores: tons de vermelho e vinho. Elementos/props de cena: pétalas de rosa vermelha, velas acesas desfocadas ao fundo. Clima geral: romântico, intimista, iluminação quente e noturna.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -5013,7 +5013,7 @@
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
 Tema visual: Dia das Crianças. Paleta de cores: tons pastéis vibrantes (amarelo, azul-bebê, rosa-claro). Elementos/props de cena: pequenos balões desfocados ao fundo, ambiente lúdico. Clima geral: leve, alegre e descontraído.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -5069,7 +5069,7 @@
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
 Tema visual: Dia das Crianças. Paleta de cores: tons pastéis vibrantes (amarelo, azul-bebê, rosa-claro). Elementos/props de cena: pequenos balões desfocados ao fundo, ambiente lúdico. Clima geral: leve, alegre e descontraído.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto) — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -5121,7 +5121,7 @@
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
 Tema visual: Dia das Crianças. Paleta de cores: tons pastéis vibrantes (amarelo, azul-bebê, rosa-claro). Elementos/props de cena: pequenos balões desfocados ao fundo, ambiente lúdico. Clima geral: leve, alegre e descontraído.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -5177,7 +5177,7 @@
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
 Tema visual: Dia das Crianças. Paleta de cores: tons pastéis vibrantes (amarelo, azul-bebê, rosa-claro). Elementos/props de cena: pequenos balões desfocados ao fundo, ambiente lúdico. Clima geral: leve, alegre e descontraído.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -5229,7 +5229,7 @@
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
 Tema visual: Dia das Crianças. Paleta de cores: tons pastéis vibrantes (amarelo, azul-bebê, rosa-claro). Elementos/props de cena: pequenos balões desfocados ao fundo, ambiente lúdico. Clima geral: leve, alegre e descontraído.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -5285,7 +5285,7 @@
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
 Tema visual: Dia das Crianças. Paleta de cores: tons pastéis vibrantes (amarelo, azul-bebê, rosa-claro). Elementos/props de cena: pequenos balões desfocados ao fundo, ambiente lúdico. Clima geral: leve, alegre e descontraído.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a mão e os dedos — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -5337,7 +5337,7 @@
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
 Tema visual: Dia das Crianças. Paleta de cores: tons pastéis vibrantes (amarelo, azul-bebê, rosa-claro). Elementos/props de cena: pequenos balões desfocados ao fundo, ambiente lúdico. Clima geral: leve, alegre e descontraído.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -5393,7 +5393,7 @@
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
 Tema visual: Dia das Crianças. Paleta de cores: tons pastéis vibrantes (amarelo, azul-bebê, rosa-claro). Elementos/props de cena: pequenos balões desfocados ao fundo, ambiente lúdico. Clima geral: leve, alegre e descontraído.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -5445,7 +5445,7 @@
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
 Tema visual: Dia dos Pais. Paleta de cores: tons de azul-marinho e cinza-grafite. Elementos/props de cena: madeira escura, textura de couro ao fundo desfocado. Clima geral: sóbrio, elegante e masculino.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -5501,7 +5501,7 @@
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
 Tema visual: Dia dos Pais. Paleta de cores: tons de azul-marinho e cinza-grafite. Elementos/props de cena: madeira escura, textura de couro ao fundo desfocado. Clima geral: sóbrio, elegante e masculino.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto) — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -5553,7 +5553,7 @@
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
 Tema visual: Dia dos Pais. Paleta de cores: tons de azul-marinho e cinza-grafite. Elementos/props de cena: madeira escura, textura de couro ao fundo desfocado. Clima geral: sóbrio, elegante e masculino.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -5609,7 +5609,7 @@
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
 Tema visual: Dia dos Pais. Paleta de cores: tons de azul-marinho e cinza-grafite. Elementos/props de cena: madeira escura, textura de couro ao fundo desfocado. Clima geral: sóbrio, elegante e masculino.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -5661,7 +5661,7 @@
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
 Tema visual: Dia dos Pais. Paleta de cores: tons de azul-marinho e cinza-grafite. Elementos/props de cena: madeira escura, textura de couro ao fundo desfocado. Clima geral: sóbrio, elegante e masculino.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -5717,7 +5717,7 @@
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
 Tema visual: Dia dos Pais. Paleta de cores: tons de azul-marinho e cinza-grafite. Elementos/props de cena: madeira escura, textura de couro ao fundo desfocado. Clima geral: sóbrio, elegante e masculino.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a mão e os dedos — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -5769,7 +5769,7 @@
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
 Tema visual: Dia dos Pais. Paleta de cores: tons de azul-marinho e cinza-grafite. Elementos/props de cena: madeira escura, textura de couro ao fundo desfocado. Clima geral: sóbrio, elegante e masculino.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -5825,7 +5825,7 @@
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
 Tema visual: Dia dos Pais. Paleta de cores: tons de azul-marinho e cinza-grafite. Elementos/props de cena: madeira escura, textura de couro ao fundo desfocado. Clima geral: sóbrio, elegante e masculino.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -5877,7 +5877,7 @@
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
 Tema visual: Dia Internacional da Mulher. Paleta de cores: tons de roxo e violeta. Elementos/props de cena: flor de mimosa (amarela) desfocada ao fundo. Clima geral: moderno, empoderado e sofisticado.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -5933,7 +5933,7 @@
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
 Tema visual: Dia Internacional da Mulher. Paleta de cores: tons de roxo e violeta. Elementos/props de cena: flor de mimosa (amarela) desfocada ao fundo. Clima geral: moderno, empoderado e sofisticado.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto) — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -5985,7 +5985,7 @@
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
 Tema visual: Dia Internacional da Mulher. Paleta de cores: tons de roxo e violeta. Elementos/props de cena: flor de mimosa (amarela) desfocada ao fundo. Clima geral: moderno, empoderado e sofisticado.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -6041,7 +6041,7 @@
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
 Tema visual: Dia Internacional da Mulher. Paleta de cores: tons de roxo e violeta. Elementos/props de cena: flor de mimosa (amarela) desfocada ao fundo. Clima geral: moderno, empoderado e sofisticado.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -6093,7 +6093,7 @@
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
 Tema visual: Dia Internacional da Mulher. Paleta de cores: tons de roxo e violeta. Elementos/props de cena: flor de mimosa (amarela) desfocada ao fundo. Clima geral: moderno, empoderado e sofisticado.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -6149,7 +6149,7 @@
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
 Tema visual: Dia Internacional da Mulher. Paleta de cores: tons de roxo e violeta. Elementos/props de cena: flor de mimosa (amarela) desfocada ao fundo. Clima geral: moderno, empoderado e sofisticado.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a mão e os dedos — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -6201,7 +6201,7 @@
       </c>
       <c r="H40" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
 Tema visual: Dia Internacional da Mulher. Paleta de cores: tons de roxo e violeta. Elementos/props de cena: flor de mimosa (amarela) desfocada ao fundo. Clima geral: moderno, empoderado e sofisticado.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -6257,7 +6257,7 @@
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
 Tema visual: Dia Internacional da Mulher. Paleta de cores: tons de roxo e violeta. Elementos/props de cena: flor de mimosa (amarela) desfocada ao fundo. Clima geral: moderno, empoderado e sofisticado.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -6309,7 +6309,7 @@
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
 Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -6365,7 +6365,7 @@
       </c>
       <c r="H43" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
 Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto) — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -6417,7 +6417,7 @@
       </c>
       <c r="H44" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
 Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -6473,7 +6473,7 @@
       </c>
       <c r="H45" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
 Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -6525,7 +6525,7 @@
       </c>
       <c r="H46" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
 Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -6581,7 +6581,7 @@
       </c>
       <c r="H47" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
 Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a mão e os dedos — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -6633,7 +6633,7 @@
       </c>
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
 Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -6689,7 +6689,7 @@
       </c>
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
 Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -6741,7 +6741,7 @@
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
 Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -6797,7 +6797,7 @@
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
 Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto) — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -6849,7 +6849,7 @@
       </c>
       <c r="H52" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
 Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -6905,7 +6905,7 @@
       </c>
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
 Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -6957,7 +6957,7 @@
       </c>
       <c r="H54" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
 Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -7013,7 +7013,7 @@
       </c>
       <c r="H55" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
 Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a mão e os dedos — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -7065,7 +7065,7 @@
       </c>
       <c r="H56" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
 Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -7121,7 +7121,7 @@
       </c>
       <c r="H57" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
 Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -7173,7 +7173,7 @@
       </c>
       <c r="H58" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
 Tema visual: Consciência Negra. Paleta de cores: tons terrosos e dourados. Elementos/props de cena: tecido com estampa de padronagem africana desfocado ao fundo. Clima geral: de valorização, orgulho e sofisticação.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -7229,7 +7229,7 @@
       </c>
       <c r="H59" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
 Tema visual: Consciência Negra. Paleta de cores: tons terrosos e dourados. Elementos/props de cena: tecido com estampa de padronagem africana desfocado ao fundo. Clima geral: de valorização, orgulho e sofisticação.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto) — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -7281,7 +7281,7 @@
       </c>
       <c r="H60" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
 Tema visual: Consciência Negra. Paleta de cores: tons terrosos e dourados. Elementos/props de cena: tecido com estampa de padronagem africana desfocado ao fundo. Clima geral: de valorização, orgulho e sofisticação.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -7337,7 +7337,7 @@
       </c>
       <c r="H61" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
 Tema visual: Consciência Negra. Paleta de cores: tons terrosos e dourados. Elementos/props de cena: tecido com estampa de padronagem africana desfocado ao fundo. Clima geral: de valorização, orgulho e sofisticação.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -7389,7 +7389,7 @@
       </c>
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
 Tema visual: Consciência Negra. Paleta de cores: tons terrosos e dourados. Elementos/props de cena: tecido com estampa de padronagem africana desfocado ao fundo. Clima geral: de valorização, orgulho e sofisticação.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -7445,7 +7445,7 @@
       </c>
       <c r="H63" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
 Tema visual: Consciência Negra. Paleta de cores: tons terrosos e dourados. Elementos/props de cena: tecido com estampa de padronagem africana desfocado ao fundo. Clima geral: de valorização, orgulho e sofisticação.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a mão e os dedos — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
@@ -7497,7 +7497,7 @@
       </c>
       <c r="H64" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
 Tema visual: Consciência Negra. Paleta de cores: tons terrosos e dourados. Elementos/props de cena: tecido com estampa de padronagem africana desfocado ao fundo. Clima geral: de valorização, orgulho e sofisticação.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
@@ -7553,7 +7553,7 @@
       </c>
       <c r="H65" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
 Tema visual: Consciência Negra. Paleta de cores: tons terrosos e dourados. Elementos/props de cena: tecido com estampa de padronagem africana desfocado ao fundo. Clima geral: de valorização, orgulho e sofisticação.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.

</xml_diff>

<commit_message>
Reforca fidelidade de quantidade e checagem de anatomia nos prompts (v4)
Incorpora tecnicas identificadas nos prompts da concorrencia: regra
explicita de contagem exata de pecas (nunca inventar/duplicar/completar
o conjunto) e checagem de anatomia (maos/dedos/pe) nas poses humanizadas
e lifestyle. Gera novo lote de UPDATE que mexe so em prompt_mestre,
preservando as fotos ja aprovadas no catalogo.
</commit_message>
<xml_diff>
--- a/content/Photo_Studio_TPV_Biblioteca_de_Prompts.xlsx
+++ b/content/Photo_Studio_TPV_Biblioteca_de_Prompts.xlsx
@@ -721,10 +721,10 @@
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H2" s="6" t="inlineStr">
@@ -771,10 +771,10 @@
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto) — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Garanta anatomia perfeita da orelha e do lóbulo — sem deformações, sem uma segunda orelha ou rosto fantasma aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H3" s="6" t="inlineStr">
@@ -817,10 +817,10 @@
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
@@ -863,10 +863,10 @@
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H5" s="6" t="inlineStr">
@@ -913,10 +913,10 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto) usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Garanta anatomia perfeita da orelha e do lóbulo — sem deformações, sem uma segunda orelha ou rosto fantasma aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
@@ -959,10 +959,10 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
@@ -1009,10 +1009,10 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
@@ -1055,10 +1055,10 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -1101,10 +1101,10 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
@@ -1151,10 +1151,10 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
@@ -1197,10 +1197,10 @@
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a peça em uma curva aberta e levemente assimétrica sobre a superfície, sugerindo o formato do pescoço sem formar um círculo perfeito ou fechado.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
@@ -1247,10 +1247,10 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pescoço, evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pescoço — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
@@ -1293,10 +1293,10 @@
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a peça em uma curva aberta e levemente assimétrica sobre a superfície, sugerindo o formato do pescoço sem formar um círculo perfeito ou fechado.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
@@ -1339,10 +1339,10 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a peça em uma curva aberta e levemente assimétrica sobre a superfície, sugerindo o formato do pescoço sem formar um círculo perfeito ou fechado.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
@@ -1389,10 +1389,10 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pescoço, evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em o pescoço usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
@@ -1435,10 +1435,10 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a corrente formando curvas amplas, orgânicas e assimétricas — nunca curvas espelhadas ou geométricas. Deixe o pingente (ou uma das extremidades) como ponto focal da composição, com o restante se estendendo de forma natural, como se tivesse acabado de cair sobre a superfície.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
@@ -1485,10 +1485,10 @@
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo e o decote, evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo e o decote — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
@@ -1531,10 +1531,10 @@
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a corrente formando curvas amplas, orgânicas e assimétricas — nunca curvas espelhadas ou geométricas. Deixe o pingente (ou uma das extremidades) como ponto focal da composição, com o restante se estendendo de forma natural, como se tivesse acabado de cair sobre a superfície.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
@@ -1577,10 +1577,10 @@
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a corrente formando curvas amplas, orgânicas e assimétricas — nunca curvas espelhadas ou geométricas. Deixe o pingente (ou uma das extremidades) como ponto focal da composição, com o restante se estendendo de forma natural, como se tivesse acabado de cair sobre a superfície.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -1627,10 +1627,10 @@
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo e o decote, evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em o colo e o decote usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
@@ -1673,10 +1673,10 @@
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o pingente como protagonista absoluto, com a corrente caindo ao redor em curvas orgânicas e assimétricas — nunca círculos, ovais ou formas espelhadas dos dois lados.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
@@ -1723,10 +1723,10 @@
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo, próximo ao centro do peito, evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, próximo ao centro do peito — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
@@ -1769,10 +1769,10 @@
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o pingente como protagonista absoluto, com a corrente caindo ao redor em curvas orgânicas e assimétricas — nunca círculos, ovais ou formas espelhadas dos dois lados.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
@@ -1815,10 +1815,10 @@
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o pingente como protagonista absoluto, com a corrente caindo ao redor em curvas orgânicas e assimétricas — nunca círculos, ovais ou formas espelhadas dos dois lados.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
@@ -1865,10 +1865,10 @@
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo, próximo ao centro do peito, evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em o colo, próximo ao centro do peito usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
@@ -1911,10 +1911,10 @@
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a corrente em uma curva reta a levemente ondulada, transmitindo peso e robustez — nunca curvas perfeitamente simétricas ou decorativas demais.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
@@ -1961,10 +1961,10 @@
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o peito e a base do pescoço, com estilo masculino, evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o peito e a base do pescoço, com estilo masculino — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
@@ -2007,10 +2007,10 @@
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a corrente em uma curva reta a levemente ondulada, transmitindo peso e robustez — nunca curvas perfeitamente simétricas ou decorativas demais.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr">
@@ -2053,10 +2053,10 @@
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a corrente em uma curva reta a levemente ondulada, transmitindo peso e robustez — nunca curvas perfeitamente simétricas ou decorativas demais.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H30" s="6" t="inlineStr">
@@ -2103,10 +2103,10 @@
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o peito e a base do pescoço, com estilo masculino, evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em o peito e a base do pescoço, com estilo masculino usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H31" s="6" t="inlineStr">
@@ -2149,10 +2149,10 @@
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H32" s="6" t="inlineStr">
@@ -2199,10 +2199,10 @@
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um pulso e uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou uma segunda mão aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H33" s="6" t="inlineStr">
@@ -2245,10 +2245,10 @@
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H34" s="6" t="inlineStr">
@@ -2291,10 +2291,10 @@
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H35" s="6" t="inlineStr">
@@ -2341,10 +2341,10 @@
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em o pulso usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um pulso e uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou uma segunda mão aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H36" s="6" t="inlineStr">
@@ -2387,10 +2387,10 @@
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o bracelete em pé, com o eixo central perpendicular à superfície (aproximadamente 90°) e inclinação máxima de 3° — o suficiente apenas para evitar aparência artificial de renderização. O centro de gravidade deve estar exatamente sobre o ponto de apoio, sem parecer tombado ou flutuando. A peça deve ocupar cerca de 65% da altura da imagem.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H37" s="6" t="inlineStr">
@@ -2437,10 +2437,10 @@
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso e o antebraço, evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso e o antebraço — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um pulso e uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou uma segunda mão aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H38" s="6" t="inlineStr">
@@ -2483,10 +2483,10 @@
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o bracelete em pé, com o eixo central perpendicular à superfície (aproximadamente 90°) e inclinação máxima de 3° — o suficiente apenas para evitar aparência artificial de renderização. O centro de gravidade deve estar exatamente sobre o ponto de apoio, sem parecer tombado ou flutuando. A peça deve ocupar cerca de 65% da altura da imagem.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H39" s="6" t="inlineStr">
@@ -2529,10 +2529,10 @@
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o bracelete em pé, com o eixo central perpendicular à superfície (aproximadamente 90°) e inclinação máxima de 3° — o suficiente apenas para evitar aparência artificial de renderização. O centro de gravidade deve estar exatamente sobre o ponto de apoio, sem parecer tombado ou flutuando. A peça deve ocupar cerca de 65% da altura da imagem.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H40" s="6" t="inlineStr">
@@ -2579,10 +2579,10 @@
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso e o antebraço, evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em o pulso e o antebraço usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um pulso e uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou uma segunda mão aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H41" s="6" t="inlineStr">
@@ -2625,10 +2625,10 @@
       </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H42" s="6" t="inlineStr">
@@ -2675,10 +2675,10 @@
       </c>
       <c r="G43" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a mão e os dedos — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, dedos fundidos, articulações deformadas ou uma segunda mão/braço aparecendo parcialmente no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H43" s="6" t="inlineStr">
@@ -2721,10 +2721,10 @@
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H44" s="6" t="inlineStr">
@@ -2767,10 +2767,10 @@
       </c>
       <c r="G45" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H45" s="6" t="inlineStr">
@@ -2817,10 +2817,10 @@
       </c>
       <c r="G46" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em a mão e os dedos usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, dedos fundidos, articulações deformadas ou uma segunda mão/braço aparecendo parcialmente no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H46" s="6" t="inlineStr">
@@ -2863,10 +2863,10 @@
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione as duas alianças em pé, lado a lado, uma levemente sobreposta à outra, ambas fisicamente equilibradas sobre a superfície — nunca flutuando.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H47" s="6" t="inlineStr">
@@ -2913,10 +2913,10 @@
       </c>
       <c r="G48" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas as mãos entrelaçadas, próximas ao dedo anelar, evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas as mãos entrelaçadas, próximas ao dedo anelar — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente duas mãos entrelaçadas, cada uma com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou deformados. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H48" s="6" t="inlineStr">
@@ -2959,10 +2959,10 @@
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione as duas alianças em pé, lado a lado, uma levemente sobreposta à outra, ambas fisicamente equilibradas sobre a superfície — nunca flutuando.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H49" s="6" t="inlineStr">
@@ -3005,10 +3005,10 @@
       </c>
       <c r="G50" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione as duas alianças em pé, lado a lado, uma levemente sobreposta à outra, ambas fisicamente equilibradas sobre a superfície — nunca flutuando.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H50" s="6" t="inlineStr">
@@ -3055,10 +3055,10 @@
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas as mãos entrelaçadas, próximas ao dedo anelar, evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em as mãos entrelaçadas, próximas ao dedo anelar usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente duas mãos entrelaçadas, cada uma com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou deformados. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H51" s="6" t="inlineStr">
@@ -3101,10 +3101,10 @@
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a peça formando uma curva aberta e natural, como se tivesse caído sobre a superfície — nunca um círculo perfeitamente fechado.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H52" s="6" t="inlineStr">
@@ -3151,10 +3151,10 @@
       </c>
       <c r="G53" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o tornozelo e o pé, evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o tornozelo e o pé — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um tornozelo e um pé, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras ou deformados. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H53" s="6" t="inlineStr">
@@ -3197,10 +3197,10 @@
       </c>
       <c r="G54" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a peça formando uma curva aberta e natural, como se tivesse caído sobre a superfície — nunca um círculo perfeitamente fechado.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H54" s="6" t="inlineStr">
@@ -3243,10 +3243,10 @@
       </c>
       <c r="G55" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a peça formando uma curva aberta e natural, como se tivesse caído sobre a superfície — nunca um círculo perfeitamente fechado.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H55" s="6" t="inlineStr">
@@ -3293,10 +3293,10 @@
       </c>
       <c r="G56" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o tornozelo e o pé, evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em o tornozelo e o pé usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um tornozelo e um pé, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras ou deformados. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H56" s="6" t="inlineStr">
@@ -3339,10 +3339,10 @@
       </c>
       <c r="G57" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o broche sobre uma prega de tecido, mostrando claramente o pino e o relevo frontal da peça, sem parecer flutuando.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H57" s="6" t="inlineStr">
@@ -3389,10 +3389,10 @@
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a lapela de um blazer ou prega de tecido, evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a lapela de um blazer ou prega de tecido — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H58" s="6" t="inlineStr">
@@ -3435,10 +3435,10 @@
       </c>
       <c r="G59" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o broche sobre uma prega de tecido, mostrando claramente o pino e o relevo frontal da peça, sem parecer flutuando.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H59" s="6" t="inlineStr">
@@ -3481,10 +3481,10 @@
       </c>
       <c r="G60" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o broche sobre uma prega de tecido, mostrando claramente o pino e o relevo frontal da peça, sem parecer flutuando.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H60" s="6" t="inlineStr">
@@ -3531,10 +3531,10 @@
       </c>
       <c r="G61" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a lapela de um blazer ou prega de tecido, evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em a lapela de um blazer ou prega de tecido usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H61" s="6" t="inlineStr">
@@ -3577,10 +3577,10 @@
       </c>
       <c r="G62" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Utilize exatamente as peças presentes na foto anexada, na mesma quantidade — nunca adicione, remova ou duplique nenhuma joia. Se não houver um tipo de peça na foto, não crie esse tipo de peça. Organize cada peça de acordo com seu próprio comportamento físico (colar em curvas orgânicas e assimétricas; brincos próximos entre si, mostrando a face principal), distribuindo os elementos em diferentes regiões da composição para um equilíbrio visual sofisticado, porém não perfeitamente simétrico.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H62" s="6" t="inlineStr">
@@ -3627,10 +3627,10 @@
       </c>
       <c r="G63" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pescoço, o colo e a orelha, evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pescoço, o colo e a orelha — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H63" s="6" t="inlineStr">
@@ -3673,10 +3673,10 @@
       </c>
       <c r="G64" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Utilize exatamente as peças presentes na foto anexada, na mesma quantidade — nunca adicione, remova ou duplique nenhuma joia. Se não houver um tipo de peça na foto, não crie esse tipo de peça. Organize cada peça de acordo com seu próprio comportamento físico (colar em curvas orgânicas e assimétricas; brincos próximos entre si, mostrando a face principal), distribuindo os elementos em diferentes regiões da composição para um equilíbrio visual sofisticado, porém não perfeitamente simétrico.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H64" s="6" t="inlineStr">
@@ -3719,10 +3719,10 @@
       </c>
       <c r="G65" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Utilize exatamente as peças presentes na foto anexada, na mesma quantidade — nunca adicione, remova ou duplique nenhuma joia. Se não houver um tipo de peça na foto, não crie esse tipo de peça. Organize cada peça de acordo com seu próprio comportamento físico (colar em curvas orgânicas e assimétricas; brincos próximos entre si, mostrando a face principal), distribuindo os elementos em diferentes regiões da composição para um equilíbrio visual sofisticado, porém não perfeitamente simétrico.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H65" s="6" t="inlineStr">
@@ -3769,10 +3769,10 @@
       </c>
       <c r="G66" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pescoço, o colo e a orelha, evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em o pescoço, o colo e a orelha usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H66" s="6" t="inlineStr">
@@ -3815,10 +3815,10 @@
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o relógio em pé, mostrando o mostrador de frente, com a pulseira formando uma curva aberta e natural ao redor — fisicamente equilibrado, nunca flutuando ou tombado.
 Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H67" s="6" t="inlineStr">
@@ -3865,10 +3865,10 @@
       </c>
       <c r="G68" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um pulso e uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou uma segunda mão aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H68" s="6" t="inlineStr">
@@ -3911,10 +3911,10 @@
       </c>
       <c r="G69" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o relógio em pé, mostrando o mostrador de frente, com a pulseira formando uma curva aberta e natural ao redor — fisicamente equilibrado, nunca flutuando ou tombado.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H69" s="6" t="inlineStr">
@@ -3957,10 +3957,10 @@
       </c>
       <c r="G70" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o relógio em pé, mostrando o mostrador de frente, com a pulseira formando uma curva aberta e natural ao redor — fisicamente equilibrado, nunca flutuando ou tombado.
 Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H70" s="6" t="inlineStr">
@@ -4007,10 +4007,10 @@
       </c>
       <c r="G71" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
 Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em o pulso usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um pulso e uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou uma segunda mão aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="H71" s="6" t="inlineStr">
@@ -4149,11 +4149,11 @@
       </c>
       <c r="H2" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
 Tema visual: Dia das Mães. Paleta de cores: tons de rosa suave e nude. Elementos/props de cena: flores (rosas) desfocadas ao fundo, tecido de seda rosa-claro. Clima geral: afetivo, delicado e caloroso.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I2" s="6" t="inlineStr">
@@ -4205,11 +4205,11 @@
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
 Tema visual: Dia das Mães. Paleta de cores: tons de rosa suave e nude. Elementos/props de cena: flores (rosas) desfocadas ao fundo, tecido de seda rosa-claro. Clima geral: afetivo, delicado e caloroso.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto) — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Garanta anatomia perfeita da orelha e do lóbulo — sem deformações, sem uma segunda orelha ou rosto fantasma aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr">
@@ -4257,11 +4257,11 @@
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
 Tema visual: Dia das Mães. Paleta de cores: tons de rosa suave e nude. Elementos/props de cena: flores (rosas) desfocadas ao fundo, tecido de seda rosa-claro. Clima geral: afetivo, delicado e caloroso.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
@@ -4313,11 +4313,11 @@
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
 Tema visual: Dia das Mães. Paleta de cores: tons de rosa suave e nude. Elementos/props de cena: flores (rosas) desfocadas ao fundo, tecido de seda rosa-claro. Clima geral: afetivo, delicado e caloroso.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
@@ -4365,11 +4365,11 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
 Tema visual: Dia das Mães. Paleta de cores: tons de rosa suave e nude. Elementos/props de cena: flores (rosas) desfocadas ao fundo, tecido de seda rosa-claro. Clima geral: afetivo, delicado e caloroso.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
@@ -4421,11 +4421,11 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
 Tema visual: Dia das Mães. Paleta de cores: tons de rosa suave e nude. Elementos/props de cena: flores (rosas) desfocadas ao fundo, tecido de seda rosa-claro. Clima geral: afetivo, delicado e caloroso.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a mão e os dedos — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, dedos fundidos, articulações deformadas ou uma segunda mão/braço aparecendo parcialmente no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
@@ -4473,11 +4473,11 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
 Tema visual: Dia das Mães. Paleta de cores: tons de rosa suave e nude. Elementos/props de cena: flores (rosas) desfocadas ao fundo, tecido de seda rosa-claro. Clima geral: afetivo, delicado e caloroso.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
@@ -4529,11 +4529,11 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
 Tema visual: Dia das Mães. Paleta de cores: tons de rosa suave e nude. Elementos/props de cena: flores (rosas) desfocadas ao fundo, tecido de seda rosa-claro. Clima geral: afetivo, delicado e caloroso.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um pulso e uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou uma segunda mão aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
@@ -4581,11 +4581,11 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
 Tema visual: Dia dos Namorados. Paleta de cores: tons de vermelho e vinho. Elementos/props de cena: pétalas de rosa vermelha, velas acesas desfocadas ao fundo. Clima geral: romântico, intimista, iluminação quente e noturna.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
@@ -4637,11 +4637,11 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
 Tema visual: Dia dos Namorados. Paleta de cores: tons de vermelho e vinho. Elementos/props de cena: pétalas de rosa vermelha, velas acesas desfocadas ao fundo. Clima geral: romântico, intimista, iluminação quente e noturna.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto) — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Garanta anatomia perfeita da orelha e do lóbulo — sem deformações, sem uma segunda orelha ou rosto fantasma aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
@@ -4689,11 +4689,11 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
 Tema visual: Dia dos Namorados. Paleta de cores: tons de vermelho e vinho. Elementos/props de cena: pétalas de rosa vermelha, velas acesas desfocadas ao fundo. Clima geral: romântico, intimista, iluminação quente e noturna.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
@@ -4745,11 +4745,11 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
 Tema visual: Dia dos Namorados. Paleta de cores: tons de vermelho e vinho. Elementos/props de cena: pétalas de rosa vermelha, velas acesas desfocadas ao fundo. Clima geral: romântico, intimista, iluminação quente e noturna.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
@@ -4797,11 +4797,11 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
 Tema visual: Dia dos Namorados. Paleta de cores: tons de vermelho e vinho. Elementos/props de cena: pétalas de rosa vermelha, velas acesas desfocadas ao fundo. Clima geral: romântico, intimista, iluminação quente e noturna.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
@@ -4853,11 +4853,11 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
 Tema visual: Dia dos Namorados. Paleta de cores: tons de vermelho e vinho. Elementos/props de cena: pétalas de rosa vermelha, velas acesas desfocadas ao fundo. Clima geral: romântico, intimista, iluminação quente e noturna.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a mão e os dedos — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, dedos fundidos, articulações deformadas ou uma segunda mão/braço aparecendo parcialmente no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
@@ -4905,11 +4905,11 @@
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
 Tema visual: Dia dos Namorados. Paleta de cores: tons de vermelho e vinho. Elementos/props de cena: pétalas de rosa vermelha, velas acesas desfocadas ao fundo. Clima geral: romântico, intimista, iluminação quente e noturna.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
@@ -4961,11 +4961,11 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
 Tema visual: Dia dos Namorados. Paleta de cores: tons de vermelho e vinho. Elementos/props de cena: pétalas de rosa vermelha, velas acesas desfocadas ao fundo. Clima geral: romântico, intimista, iluminação quente e noturna.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um pulso e uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou uma segunda mão aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
@@ -5013,11 +5013,11 @@
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
 Tema visual: Dia das Crianças. Paleta de cores: tons pastéis vibrantes (amarelo, azul-bebê, rosa-claro). Elementos/props de cena: pequenos balões desfocados ao fundo, ambiente lúdico. Clima geral: leve, alegre e descontraído.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
@@ -5069,11 +5069,11 @@
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
 Tema visual: Dia das Crianças. Paleta de cores: tons pastéis vibrantes (amarelo, azul-bebê, rosa-claro). Elementos/props de cena: pequenos balões desfocados ao fundo, ambiente lúdico. Clima geral: leve, alegre e descontraído.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto) — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Garanta anatomia perfeita da orelha e do lóbulo — sem deformações, sem uma segunda orelha ou rosto fantasma aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr">
@@ -5121,11 +5121,11 @@
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
 Tema visual: Dia das Crianças. Paleta de cores: tons pastéis vibrantes (amarelo, azul-bebê, rosa-claro). Elementos/props de cena: pequenos balões desfocados ao fundo, ambiente lúdico. Clima geral: leve, alegre e descontraído.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr">
@@ -5177,11 +5177,11 @@
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
 Tema visual: Dia das Crianças. Paleta de cores: tons pastéis vibrantes (amarelo, azul-bebê, rosa-claro). Elementos/props de cena: pequenos balões desfocados ao fundo, ambiente lúdico. Clima geral: leve, alegre e descontraído.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr">
@@ -5229,11 +5229,11 @@
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
 Tema visual: Dia das Crianças. Paleta de cores: tons pastéis vibrantes (amarelo, azul-bebê, rosa-claro). Elementos/props de cena: pequenos balões desfocados ao fundo, ambiente lúdico. Clima geral: leve, alegre e descontraído.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
@@ -5285,11 +5285,11 @@
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
 Tema visual: Dia das Crianças. Paleta de cores: tons pastéis vibrantes (amarelo, azul-bebê, rosa-claro). Elementos/props de cena: pequenos balões desfocados ao fundo, ambiente lúdico. Clima geral: leve, alegre e descontraído.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a mão e os dedos — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, dedos fundidos, articulações deformadas ou uma segunda mão/braço aparecendo parcialmente no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr">
@@ -5337,11 +5337,11 @@
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
 Tema visual: Dia das Crianças. Paleta de cores: tons pastéis vibrantes (amarelo, azul-bebê, rosa-claro). Elementos/props de cena: pequenos balões desfocados ao fundo, ambiente lúdico. Clima geral: leve, alegre e descontraído.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr">
@@ -5393,11 +5393,11 @@
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
 Tema visual: Dia das Crianças. Paleta de cores: tons pastéis vibrantes (amarelo, azul-bebê, rosa-claro). Elementos/props de cena: pequenos balões desfocados ao fundo, ambiente lúdico. Clima geral: leve, alegre e descontraído.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um pulso e uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou uma segunda mão aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
@@ -5445,11 +5445,11 @@
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
 Tema visual: Dia dos Pais. Paleta de cores: tons de azul-marinho e cinza-grafite. Elementos/props de cena: madeira escura, textura de couro ao fundo desfocado. Clima geral: sóbrio, elegante e masculino.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
@@ -5501,11 +5501,11 @@
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
 Tema visual: Dia dos Pais. Paleta de cores: tons de azul-marinho e cinza-grafite. Elementos/props de cena: madeira escura, textura de couro ao fundo desfocado. Clima geral: sóbrio, elegante e masculino.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto) — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Garanta anatomia perfeita da orelha e do lóbulo — sem deformações, sem uma segunda orelha ou rosto fantasma aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
@@ -5553,11 +5553,11 @@
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
 Tema visual: Dia dos Pais. Paleta de cores: tons de azul-marinho e cinza-grafite. Elementos/props de cena: madeira escura, textura de couro ao fundo desfocado. Clima geral: sóbrio, elegante e masculino.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
@@ -5609,11 +5609,11 @@
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
 Tema visual: Dia dos Pais. Paleta de cores: tons de azul-marinho e cinza-grafite. Elementos/props de cena: madeira escura, textura de couro ao fundo desfocado. Clima geral: sóbrio, elegante e masculino.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
@@ -5661,11 +5661,11 @@
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
 Tema visual: Dia dos Pais. Paleta de cores: tons de azul-marinho e cinza-grafite. Elementos/props de cena: madeira escura, textura de couro ao fundo desfocado. Clima geral: sóbrio, elegante e masculino.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
@@ -5717,11 +5717,11 @@
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
 Tema visual: Dia dos Pais. Paleta de cores: tons de azul-marinho e cinza-grafite. Elementos/props de cena: madeira escura, textura de couro ao fundo desfocado. Clima geral: sóbrio, elegante e masculino.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a mão e os dedos — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, dedos fundidos, articulações deformadas ou uma segunda mão/braço aparecendo parcialmente no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
@@ -5769,11 +5769,11 @@
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
 Tema visual: Dia dos Pais. Paleta de cores: tons de azul-marinho e cinza-grafite. Elementos/props de cena: madeira escura, textura de couro ao fundo desfocado. Clima geral: sóbrio, elegante e masculino.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
@@ -5825,11 +5825,11 @@
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
 Tema visual: Dia dos Pais. Paleta de cores: tons de azul-marinho e cinza-grafite. Elementos/props de cena: madeira escura, textura de couro ao fundo desfocado. Clima geral: sóbrio, elegante e masculino.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um pulso e uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou uma segunda mão aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
@@ -5877,11 +5877,11 @@
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
 Tema visual: Dia Internacional da Mulher. Paleta de cores: tons de roxo e violeta. Elementos/props de cena: flor de mimosa (amarela) desfocada ao fundo. Clima geral: moderno, empoderado e sofisticado.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr">
@@ -5933,11 +5933,11 @@
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
 Tema visual: Dia Internacional da Mulher. Paleta de cores: tons de roxo e violeta. Elementos/props de cena: flor de mimosa (amarela) desfocada ao fundo. Clima geral: moderno, empoderado e sofisticado.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto) — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Garanta anatomia perfeita da orelha e do lóbulo — sem deformações, sem uma segunda orelha ou rosto fantasma aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
@@ -5985,11 +5985,11 @@
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
 Tema visual: Dia Internacional da Mulher. Paleta de cores: tons de roxo e violeta. Elementos/props de cena: flor de mimosa (amarela) desfocada ao fundo. Clima geral: moderno, empoderado e sofisticado.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
@@ -6041,11 +6041,11 @@
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
 Tema visual: Dia Internacional da Mulher. Paleta de cores: tons de roxo e violeta. Elementos/props de cena: flor de mimosa (amarela) desfocada ao fundo. Clima geral: moderno, empoderado e sofisticado.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
@@ -6093,11 +6093,11 @@
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
 Tema visual: Dia Internacional da Mulher. Paleta de cores: tons de roxo e violeta. Elementos/props de cena: flor de mimosa (amarela) desfocada ao fundo. Clima geral: moderno, empoderado e sofisticado.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
@@ -6149,11 +6149,11 @@
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
 Tema visual: Dia Internacional da Mulher. Paleta de cores: tons de roxo e violeta. Elementos/props de cena: flor de mimosa (amarela) desfocada ao fundo. Clima geral: moderno, empoderado e sofisticado.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a mão e os dedos — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, dedos fundidos, articulações deformadas ou uma segunda mão/braço aparecendo parcialmente no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr">
@@ -6201,11 +6201,11 @@
       </c>
       <c r="H40" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
 Tema visual: Dia Internacional da Mulher. Paleta de cores: tons de roxo e violeta. Elementos/props de cena: flor de mimosa (amarela) desfocada ao fundo. Clima geral: moderno, empoderado e sofisticado.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr">
@@ -6257,11 +6257,11 @@
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
 Tema visual: Dia Internacional da Mulher. Paleta de cores: tons de roxo e violeta. Elementos/props de cena: flor de mimosa (amarela) desfocada ao fundo. Clima geral: moderno, empoderado e sofisticado.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um pulso e uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou uma segunda mão aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr">
@@ -6309,11 +6309,11 @@
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
 Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr">
@@ -6365,11 +6365,11 @@
       </c>
       <c r="H43" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
 Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto) — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Garanta anatomia perfeita da orelha e do lóbulo — sem deformações, sem uma segunda orelha ou rosto fantasma aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr">
@@ -6417,11 +6417,11 @@
       </c>
       <c r="H44" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
 Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I44" s="6" t="inlineStr">
@@ -6473,11 +6473,11 @@
       </c>
       <c r="H45" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
 Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I45" s="6" t="inlineStr">
@@ -6525,11 +6525,11 @@
       </c>
       <c r="H46" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
 Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I46" s="6" t="inlineStr">
@@ -6581,11 +6581,11 @@
       </c>
       <c r="H47" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
 Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a mão e os dedos — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, dedos fundidos, articulações deformadas ou uma segunda mão/braço aparecendo parcialmente no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I47" s="6" t="inlineStr">
@@ -6633,11 +6633,11 @@
       </c>
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
 Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr">
@@ -6689,11 +6689,11 @@
       </c>
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
 Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um pulso e uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou uma segunda mão aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr">
@@ -6741,11 +6741,11 @@
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
 Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr">
@@ -6797,11 +6797,11 @@
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
 Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto) — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Garanta anatomia perfeita da orelha e do lóbulo — sem deformações, sem uma segunda orelha ou rosto fantasma aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr">
@@ -6849,11 +6849,11 @@
       </c>
       <c r="H52" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
 Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I52" s="6" t="inlineStr">
@@ -6905,11 +6905,11 @@
       </c>
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
 Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I53" s="6" t="inlineStr">
@@ -6957,11 +6957,11 @@
       </c>
       <c r="H54" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
 Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I54" s="6" t="inlineStr">
@@ -7013,11 +7013,11 @@
       </c>
       <c r="H55" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
 Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a mão e os dedos — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, dedos fundidos, articulações deformadas ou uma segunda mão/braço aparecendo parcialmente no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I55" s="6" t="inlineStr">
@@ -7065,11 +7065,11 @@
       </c>
       <c r="H56" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
 Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I56" s="6" t="inlineStr">
@@ -7121,11 +7121,11 @@
       </c>
       <c r="H57" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
 Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um pulso e uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou uma segunda mão aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I57" s="6" t="inlineStr">
@@ -7173,11 +7173,11 @@
       </c>
       <c r="H58" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
 Tema visual: Consciência Negra. Paleta de cores: tons terrosos e dourados. Elementos/props de cena: tecido com estampa de padronagem africana desfocado ao fundo. Clima geral: de valorização, orgulho e sofisticação.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I58" s="6" t="inlineStr">
@@ -7229,11 +7229,11 @@
       </c>
       <c r="H59" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
 Tema visual: Consciência Negra. Paleta de cores: tons terrosos e dourados. Elementos/props de cena: tecido com estampa de padronagem africana desfocado ao fundo. Clima geral: de valorização, orgulho e sofisticação.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto) — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Garanta anatomia perfeita da orelha e do lóbulo — sem deformações, sem uma segunda orelha ou rosto fantasma aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I59" s="6" t="inlineStr">
@@ -7281,11 +7281,11 @@
       </c>
       <c r="H60" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
 Tema visual: Consciência Negra. Paleta de cores: tons terrosos e dourados. Elementos/props de cena: tecido com estampa de padronagem africana desfocado ao fundo. Clima geral: de valorização, orgulho e sofisticação.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I60" s="6" t="inlineStr">
@@ -7337,11 +7337,11 @@
       </c>
       <c r="H61" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
 Tema visual: Consciência Negra. Paleta de cores: tons terrosos e dourados. Elementos/props de cena: tecido com estampa de padronagem africana desfocado ao fundo. Clima geral: de valorização, orgulho e sofisticação.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I61" s="6" t="inlineStr">
@@ -7389,11 +7389,11 @@
       </c>
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
 Tema visual: Consciência Negra. Paleta de cores: tons terrosos e dourados. Elementos/props de cena: tecido com estampa de padronagem africana desfocado ao fundo. Clima geral: de valorização, orgulho e sofisticação.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I62" s="6" t="inlineStr">
@@ -7445,11 +7445,11 @@
       </c>
       <c r="H63" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
 Tema visual: Consciência Negra. Paleta de cores: tons terrosos e dourados. Elementos/props de cena: tecido com estampa de padronagem africana desfocado ao fundo. Clima geral: de valorização, orgulho e sofisticação.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a mão e os dedos — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, dedos fundidos, articulações deformadas ou uma segunda mão/braço aparecendo parcialmente no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr">
@@ -7497,11 +7497,11 @@
       </c>
       <c r="H64" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
 Tema visual: Consciência Negra. Paleta de cores: tons terrosos e dourados. Elementos/props de cena: tecido com estampa de padronagem africana desfocado ao fundo. Clima geral: de valorização, orgulho e sofisticação.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I64" s="6" t="inlineStr">
@@ -7553,11 +7553,11 @@
       </c>
       <c r="H65" s="6" t="inlineStr">
         <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
 Tema visual: Consciência Negra. Paleta de cores: tons terrosos e dourados. Elementos/props de cena: tecido com estampa de padronagem africana desfocado ao fundo. Clima geral: de valorização, orgulho e sofisticação.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme que a peça gerada corresponde exatamente, em quantidade e em detalhes, à peça da imagem original. Formato final da imagem: 3:4 (vertical).</t>
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um pulso e uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou uma segunda mão aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
       <c r="I65" s="6" t="inlineStr">

</xml_diff>

<commit_message>
v5: remove Relogio, reduz Datas Comemorativas a 5 fotos/data e adiciona Expositores
- Remove a categoria Relogio de todos os dicionarios do gerador.
- Datas Comemorativas: mantem so 7 datas (tira Dia das Criancas), 5 fotos
  por data variando peca/cenario em vez do grid fixo de 8.
- Nova aba/categoria Expositores: 10 prompts still de joia sobre suporte
  de exibicao (busto, mao, orelha, correntes), reaproveitando os cenarios
  ja existentes (still branco, sombra editorial, textura).
- scripts/gen_migration_v5.py gera o DELETE (relogio + datas antigas) e
  os INSERT da nova estrutura, separado do fluxo normal de UPDATE de
  prompt_mestre usado pelas revisoes de texto.
</commit_message>
<xml_diff>
--- a/content/Photo_Studio_TPV_Biblioteca_de_Prompts.xlsx
+++ b/content/Photo_Studio_TPV_Biblioteca_de_Prompts.xlsx
@@ -10,10 +10,12 @@
     <sheet name="Instruções" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Evergreen" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Datas Comemorativas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Expositores" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Evergreen'!$A$1:$K$71</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Datas Comemorativas'!$A$1:$L$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Evergreen'!$A$1:$K$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Datas Comemorativas'!$A$1:$L$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Expositores'!$A$1:$K$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -621,7 +623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K71"/>
+  <dimension ref="A1:K66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3788,246 +3790,8 @@
       <c r="J66" s="6" t="inlineStr"/>
       <c r="K66" s="6" t="inlineStr"/>
     </row>
-    <row r="67" ht="130" customHeight="1">
-      <c r="A67" s="6" t="n">
-        <v>66</v>
-      </c>
-      <c r="B67" s="6" t="inlineStr">
-        <is>
-          <t>Relógio</t>
-        </is>
-      </c>
-      <c r="C67" s="6" t="inlineStr">
-        <is>
-          <t>Still Branco (Packshot)</t>
-        </is>
-      </c>
-      <c r="D67" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E67" s="6" t="inlineStr"/>
-      <c r="F67" s="6" t="inlineStr">
-        <is>
-          <t>relogio_still-branco-packshot</t>
-        </is>
-      </c>
-      <c r="G67" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: Posicione o relógio em pé, mostrando o mostrador de frente, com a pulseira formando uma curva aberta e natural ao redor — fisicamente equilibrado, nunca flutuando ou tombado.
-Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="H67" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="I67" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="J67" s="6" t="inlineStr"/>
-      <c r="K67" s="6" t="inlineStr"/>
-    </row>
-    <row r="68" ht="130" customHeight="1">
-      <c r="A68" s="6" t="n">
-        <v>67</v>
-      </c>
-      <c r="B68" s="6" t="inlineStr">
-        <is>
-          <t>Relógio</t>
-        </is>
-      </c>
-      <c r="C68" s="6" t="inlineStr">
-        <is>
-          <t>Still Humanizado</t>
-        </is>
-      </c>
-      <c r="D68" s="6" t="inlineStr">
-        <is>
-          <t>Sim (parte do corpo, sem rosto)</t>
-        </is>
-      </c>
-      <c r="E68" s="6" t="inlineStr">
-        <is>
-          <t>Mulher adulta (30-45), pele morena | Homem adulto (35-50), pele clara | Mulher idosa (60+), pele negra</t>
-        </is>
-      </c>
-      <c r="F68" s="6" t="inlineStr">
-        <is>
-          <t>relogio_still-humanizado</t>
-        </is>
-      </c>
-      <c r="G68" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
-Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um pulso e uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou uma segunda mão aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="H68" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="I68" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="J68" s="6" t="inlineStr"/>
-      <c r="K68" s="6" t="inlineStr"/>
-    </row>
-    <row r="69" ht="130" customHeight="1">
-      <c r="A69" s="6" t="n">
-        <v>68</v>
-      </c>
-      <c r="B69" s="6" t="inlineStr">
-        <is>
-          <t>Relógio</t>
-        </is>
-      </c>
-      <c r="C69" s="6" t="inlineStr">
-        <is>
-          <t>Still com Sombra Editorial</t>
-        </is>
-      </c>
-      <c r="D69" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E69" s="6" t="inlineStr"/>
-      <c r="F69" s="6" t="inlineStr">
-        <is>
-          <t>relogio_still-com-sombra-editorial</t>
-        </is>
-      </c>
-      <c r="G69" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: Posicione o relógio em pé, mostrando o mostrador de frente, com a pulseira formando uma curva aberta e natural ao redor — fisicamente equilibrado, nunca flutuando ou tombado.
-Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="H69" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="I69" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="J69" s="6" t="inlineStr"/>
-      <c r="K69" s="6" t="inlineStr"/>
-    </row>
-    <row r="70" ht="130" customHeight="1">
-      <c r="A70" s="6" t="n">
-        <v>69</v>
-      </c>
-      <c r="B70" s="6" t="inlineStr">
-        <is>
-          <t>Relógio</t>
-        </is>
-      </c>
-      <c r="C70" s="6" t="inlineStr">
-        <is>
-          <t>Still em Superfície Texturizada</t>
-        </is>
-      </c>
-      <c r="D70" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E70" s="6" t="inlineStr"/>
-      <c r="F70" s="6" t="inlineStr">
-        <is>
-          <t>relogio_still-em-superficie-texturizada</t>
-        </is>
-      </c>
-      <c r="G70" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: Posicione o relógio em pé, mostrando o mostrador de frente, com a pulseira formando uma curva aberta e natural ao redor — fisicamente equilibrado, nunca flutuando ou tombado.
-Fotografia still editorial sobre uma superfície de linho bege, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="H70" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="I70" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="J70" s="6" t="inlineStr"/>
-      <c r="K70" s="6" t="inlineStr"/>
-    </row>
-    <row r="71" ht="130" customHeight="1">
-      <c r="A71" s="6" t="n">
-        <v>70</v>
-      </c>
-      <c r="B71" s="6" t="inlineStr">
-        <is>
-          <t>Relógio</t>
-        </is>
-      </c>
-      <c r="C71" s="6" t="inlineStr">
-        <is>
-          <t>Lifestyle com Modelo</t>
-        </is>
-      </c>
-      <c r="D71" s="6" t="inlineStr">
-        <is>
-          <t>Sim (parte do corpo, sem rosto)</t>
-        </is>
-      </c>
-      <c r="E71" s="6" t="inlineStr">
-        <is>
-          <t>Mulher adulta (30-45), pele morena | Homem adulto (35-50), pele clara | Mulher idosa (60+), pele negra</t>
-        </is>
-      </c>
-      <c r="F71" s="6" t="inlineStr">
-        <is>
-          <t>relogio_lifestyle-com-modelo</t>
-        </is>
-      </c>
-      <c r="G71" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
-Fotografia lifestyle editorial para redes sociais e e-commerce. Enquadramento fechado o suficiente para não mostrar o rosto da modelo — foco em o pulso usando a peça de forma natural, em um gesto espontâneo do dia a dia, compatível com o tipo de peça. Iluminação natural suave, como luz de uma janela lateral ampla, sem fonte artificial. Fundo desfocado (profundidade de campo rasa), sugerindo um ambiente interno elegante e minimalista, sem elementos que disputem atenção com a joia. Tons neutros e quentes (branco, off-white, bege). A peça deve permanecer perfeitamente nítida e iluminada, com reflexos naturais e fisicamente corretos no metal.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um pulso e uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou uma segunda mão aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="H71" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="I71" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="J71" s="6" t="inlineStr"/>
-      <c r="K71" s="6" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K71"/>
+  <autoFilter ref="A1:K66"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4038,7 +3802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L65"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4123,7 +3887,7 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>Dia das Mães</t>
+          <t>Natal</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
@@ -4144,10 +3908,442 @@
       <c r="F2" s="6" t="inlineStr"/>
       <c r="G2" s="6" t="inlineStr">
         <is>
+          <t>natal_brinco_still-com-tema</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
+Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
+Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="K2" s="6" t="inlineStr"/>
+      <c r="L2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3" ht="140" customHeight="1">
+      <c r="A3" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Natal</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Brinco</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Lifestyle com Tema</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Sim (parte do corpo, sem rosto)</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>natal_brinco_lifestyle-com-tema</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
+Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
+Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto) — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Garanta anatomia perfeita da orelha e do lóbulo — sem deformações, sem uma segunda orelha ou rosto fantasma aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="K3" s="6" t="inlineStr"/>
+      <c r="L3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4" ht="140" customHeight="1">
+      <c r="A4" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Natal</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Colar</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Still com Tema</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr"/>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>natal_colar_still-com-tema</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
+Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
+Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="K4" s="6" t="inlineStr"/>
+      <c r="L4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5" ht="140" customHeight="1">
+      <c r="A5" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Natal</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Colar</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Lifestyle com Tema</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Sim (parte do corpo, sem rosto)</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>natal_colar_lifestyle-com-tema</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
+Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
+Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr"/>
+      <c r="L5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6" ht="140" customHeight="1">
+      <c r="A6" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Natal</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Anel</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Still com Tema</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr"/>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>natal_anel_still-com-tema</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
+Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
+Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="K6" s="6" t="inlineStr"/>
+      <c r="L6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7" ht="140" customHeight="1">
+      <c r="A7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Dia das Mães</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Anel</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Lifestyle com Tema</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Sim (parte do corpo, sem rosto)</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>dia-das-maes_anel_lifestyle-com-tema</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
+Tema visual: Dia das Mães. Paleta de cores: tons de rosa suave e nude. Elementos/props de cena: flores (rosas) desfocadas ao fundo, tecido de seda rosa-claro. Clima geral: afetivo, delicado e caloroso.
+Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a mão e os dedos — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, dedos fundidos, articulações deformadas ou uma segunda mão/braço aparecendo parcialmente no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="inlineStr"/>
+      <c r="L7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8" ht="140" customHeight="1">
+      <c r="A8" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Dia das Mães</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Pulseira</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Still com Tema</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr"/>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>dia-das-maes_pulseira_still-com-tema</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
+Tema visual: Dia das Mães. Paleta de cores: tons de rosa suave e nude. Elementos/props de cena: flores (rosas) desfocadas ao fundo, tecido de seda rosa-claro. Clima geral: afetivo, delicado e caloroso.
+Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="K8" s="6" t="inlineStr"/>
+      <c r="L8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9" ht="140" customHeight="1">
+      <c r="A9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Dia das Mães</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Pulseira</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Lifestyle com Tema</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Sim (parte do corpo, sem rosto)</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>dia-das-maes_pulseira_lifestyle-com-tema</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
+Tema visual: Dia das Mães. Paleta de cores: tons de rosa suave e nude. Elementos/props de cena: flores (rosas) desfocadas ao fundo, tecido de seda rosa-claro. Clima geral: afetivo, delicado e caloroso.
+Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um pulso e uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou uma segunda mão aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="inlineStr"/>
+      <c r="L9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10" ht="140" customHeight="1">
+      <c r="A10" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Dia das Mães</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Brinco</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Still com Tema</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr"/>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
           <t>dia-das-maes_brinco_still-com-tema</t>
         </is>
       </c>
-      <c r="H2" s="6" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
@@ -4156,54 +4352,54 @@
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
-      <c r="I2" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J2" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K2" s="6" t="inlineStr"/>
-      <c r="L2" s="6" t="inlineStr"/>
-    </row>
-    <row r="3" ht="140" customHeight="1">
-      <c r="A3" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="inlineStr"/>
+      <c r="L10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11" ht="140" customHeight="1">
+      <c r="A11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Dia das Mães</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Brinco</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>Lifestyle com Tema</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>Sim (parte do corpo, sem rosto)</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>dia-das-maes_brinco_lifestyle-com-tema</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
@@ -4212,438 +4408,6 @@
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Garanta anatomia perfeita da orelha e do lóbulo — sem deformações, sem uma segunda orelha ou rosto fantasma aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
-      <c r="I3" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J3" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K3" s="6" t="inlineStr"/>
-      <c r="L3" s="6" t="inlineStr"/>
-    </row>
-    <row r="4" ht="140" customHeight="1">
-      <c r="A4" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>Dia das Mães</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Colar</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>Still com Tema</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>dia-das-maes_colar_still-com-tema</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
-Tema visual: Dia das Mães. Paleta de cores: tons de rosa suave e nude. Elementos/props de cena: flores (rosas) desfocadas ao fundo, tecido de seda rosa-claro. Clima geral: afetivo, delicado e caloroso.
-Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I4" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J4" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K4" s="6" t="inlineStr"/>
-      <c r="L4" s="6" t="inlineStr"/>
-    </row>
-    <row r="5" ht="140" customHeight="1">
-      <c r="A5" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Dia das Mães</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>Colar</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>Lifestyle com Tema</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>Sim (parte do corpo, sem rosto)</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>dia-das-maes_colar_lifestyle-com-tema</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
-Tema visual: Dia das Mães. Paleta de cores: tons de rosa suave e nude. Elementos/props de cena: flores (rosas) desfocadas ao fundo, tecido de seda rosa-claro. Clima geral: afetivo, delicado e caloroso.
-Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I5" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J5" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K5" s="6" t="inlineStr"/>
-      <c r="L5" s="6" t="inlineStr"/>
-    </row>
-    <row r="6" ht="140" customHeight="1">
-      <c r="A6" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Dia das Mães</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>Anel</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>Still com Tema</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>dia-das-maes_anel_still-com-tema</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
-Tema visual: Dia das Mães. Paleta de cores: tons de rosa suave e nude. Elementos/props de cena: flores (rosas) desfocadas ao fundo, tecido de seda rosa-claro. Clima geral: afetivo, delicado e caloroso.
-Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J6" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K6" s="6" t="inlineStr"/>
-      <c r="L6" s="6" t="inlineStr"/>
-    </row>
-    <row r="7" ht="140" customHeight="1">
-      <c r="A7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Dia das Mães</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Anel</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>Lifestyle com Tema</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>Sim (parte do corpo, sem rosto)</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>dia-das-maes_anel_lifestyle-com-tema</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
-Tema visual: Dia das Mães. Paleta de cores: tons de rosa suave e nude. Elementos/props de cena: flores (rosas) desfocadas ao fundo, tecido de seda rosa-claro. Clima geral: afetivo, delicado e caloroso.
-Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a mão e os dedos — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, dedos fundidos, articulações deformadas ou uma segunda mão/braço aparecendo parcialmente no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K7" s="6" t="inlineStr"/>
-      <c r="L7" s="6" t="inlineStr"/>
-    </row>
-    <row r="8" ht="140" customHeight="1">
-      <c r="A8" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Dia das Mães</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>Pulseira</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>Still com Tema</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr"/>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>dia-das-maes_pulseira_still-com-tema</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
-Tema visual: Dia das Mães. Paleta de cores: tons de rosa suave e nude. Elementos/props de cena: flores (rosas) desfocadas ao fundo, tecido de seda rosa-claro. Clima geral: afetivo, delicado e caloroso.
-Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J8" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K8" s="6" t="inlineStr"/>
-      <c r="L8" s="6" t="inlineStr"/>
-    </row>
-    <row r="9" ht="140" customHeight="1">
-      <c r="A9" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Dia das Mães</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>Pulseira</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Lifestyle com Tema</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>Sim (parte do corpo, sem rosto)</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>dia-das-maes_pulseira_lifestyle-com-tema</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
-Tema visual: Dia das Mães. Paleta de cores: tons de rosa suave e nude. Elementos/props de cena: flores (rosas) desfocadas ao fundo, tecido de seda rosa-claro. Clima geral: afetivo, delicado e caloroso.
-Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um pulso e uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou uma segunda mão aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J9" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K9" s="6" t="inlineStr"/>
-      <c r="L9" s="6" t="inlineStr"/>
-    </row>
-    <row r="10" ht="140" customHeight="1">
-      <c r="A10" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Dia dos Namorados</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>Brinco</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>Still com Tema</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr"/>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>dia-dos-namorados_brinco_still-com-tema</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
-Tema visual: Dia dos Namorados. Paleta de cores: tons de vermelho e vinho. Elementos/props de cena: pétalas de rosa vermelha, velas acesas desfocadas ao fundo. Clima geral: romântico, intimista, iluminação quente e noturna.
-Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I10" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J10" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K10" s="6" t="inlineStr"/>
-      <c r="L10" s="6" t="inlineStr"/>
-    </row>
-    <row r="11" ht="140" customHeight="1">
-      <c r="A11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>Dia dos Namorados</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>Brinco</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>Lifestyle com Tema</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>Sim (parte do corpo, sem rosto)</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>dia-dos-namorados_brinco_lifestyle-com-tema</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
-Tema visual: Dia dos Namorados. Paleta de cores: tons de vermelho e vinho. Elementos/props de cena: pétalas de rosa vermelha, velas acesas desfocadas ao fundo. Clima geral: romântico, intimista, iluminação quente e noturna.
-Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto) — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Garanta anatomia perfeita da orelha e do lóbulo — sem deformações, sem uma segunda orelha ou rosto fantasma aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
           <t>3:4 (vertical)</t>
@@ -4931,7 +4695,7 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Dia dos Namorados</t>
+          <t>Black Friday</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -4956,14 +4720,14 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>dia-dos-namorados_pulseira_lifestyle-com-tema</t>
+          <t>black-friday_pulseira_lifestyle-com-tema</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
           <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
-Tema visual: Dia dos Namorados. Paleta de cores: tons de vermelho e vinho. Elementos/props de cena: pétalas de rosa vermelha, velas acesas desfocadas ao fundo. Clima geral: romântico, intimista, iluminação quente e noturna.
+Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um pulso e uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou uma segunda mão aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
@@ -4987,7 +4751,7 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Dia das Crianças</t>
+          <t>Black Friday</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -5008,14 +4772,14 @@
       <c r="F18" s="6" t="inlineStr"/>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>dia-das-criancas_brinco_still-com-tema</t>
+          <t>black-friday_brinco_still-com-tema</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
           <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
-Tema visual: Dia das Crianças. Paleta de cores: tons pastéis vibrantes (amarelo, azul-bebê, rosa-claro). Elementos/props de cena: pequenos balões desfocados ao fundo, ambiente lúdico. Clima geral: leve, alegre e descontraído.
+Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
@@ -5039,7 +4803,7 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Dia das Crianças</t>
+          <t>Black Friday</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -5064,14 +4828,14 @@
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>dia-das-criancas_brinco_lifestyle-com-tema</t>
+          <t>black-friday_brinco_lifestyle-com-tema</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
           <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
-Tema visual: Dia das Crianças. Paleta de cores: tons pastéis vibrantes (amarelo, azul-bebê, rosa-claro). Elementos/props de cena: pequenos balões desfocados ao fundo, ambiente lúdico. Clima geral: leve, alegre e descontraído.
+Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto) — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Garanta anatomia perfeita da orelha e do lóbulo — sem deformações, sem uma segunda orelha ou rosto fantasma aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
@@ -5095,7 +4859,7 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Dia das Crianças</t>
+          <t>Black Friday</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -5116,14 +4880,14 @@
       <c r="F20" s="6" t="inlineStr"/>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>dia-das-criancas_colar_still-com-tema</t>
+          <t>black-friday_colar_still-com-tema</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
           <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
-Tema visual: Dia das Crianças. Paleta de cores: tons pastéis vibrantes (amarelo, azul-bebê, rosa-claro). Elementos/props de cena: pequenos balões desfocados ao fundo, ambiente lúdico. Clima geral: leve, alegre e descontraído.
+Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
@@ -5147,7 +4911,7 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Dia das Crianças</t>
+          <t>Black Friday</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -5172,14 +4936,14 @@
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>dia-das-criancas_colar_lifestyle-com-tema</t>
+          <t>black-friday_colar_lifestyle-com-tema</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
           <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
-Tema visual: Dia das Crianças. Paleta de cores: tons pastéis vibrantes (amarelo, azul-bebê, rosa-claro). Elementos/props de cena: pequenos balões desfocados ao fundo, ambiente lúdico. Clima geral: leve, alegre e descontraído.
+Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
@@ -5203,7 +4967,7 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Dia das Crianças</t>
+          <t>Dia dos Pais</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -5224,14 +4988,14 @@
       <c r="F22" s="6" t="inlineStr"/>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>dia-das-criancas_anel_still-com-tema</t>
+          <t>dia-dos-pais_anel_still-com-tema</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
           <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
-Tema visual: Dia das Crianças. Paleta de cores: tons pastéis vibrantes (amarelo, azul-bebê, rosa-claro). Elementos/props de cena: pequenos balões desfocados ao fundo, ambiente lúdico. Clima geral: leve, alegre e descontraído.
+Tema visual: Dia dos Pais. Paleta de cores: tons de azul-marinho e cinza-grafite. Elementos/props de cena: madeira escura, textura de couro ao fundo desfocado. Clima geral: sóbrio, elegante e masculino.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
@@ -5255,7 +5019,7 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Dia das Crianças</t>
+          <t>Dia dos Pais</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
@@ -5280,442 +5044,10 @@
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>dia-das-criancas_anel_lifestyle-com-tema</t>
+          <t>dia-dos-pais_anel_lifestyle-com-tema</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
-Tema visual: Dia das Crianças. Paleta de cores: tons pastéis vibrantes (amarelo, azul-bebê, rosa-claro). Elementos/props de cena: pequenos balões desfocados ao fundo, ambiente lúdico. Clima geral: leve, alegre e descontraído.
-Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a mão e os dedos — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, dedos fundidos, articulações deformadas ou uma segunda mão/braço aparecendo parcialmente no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I23" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J23" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K23" s="6" t="inlineStr"/>
-      <c r="L23" s="6" t="inlineStr"/>
-    </row>
-    <row r="24" ht="140" customHeight="1">
-      <c r="A24" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>Dia das Crianças</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>Pulseira</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>Still com Tema</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr"/>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>dia-das-criancas_pulseira_still-com-tema</t>
-        </is>
-      </c>
-      <c r="H24" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
-Tema visual: Dia das Crianças. Paleta de cores: tons pastéis vibrantes (amarelo, azul-bebê, rosa-claro). Elementos/props de cena: pequenos balões desfocados ao fundo, ambiente lúdico. Clima geral: leve, alegre e descontraído.
-Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I24" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J24" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K24" s="6" t="inlineStr"/>
-      <c r="L24" s="6" t="inlineStr"/>
-    </row>
-    <row r="25" ht="140" customHeight="1">
-      <c r="A25" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>Dia das Crianças</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>Pulseira</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>Lifestyle com Tema</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>Sim (parte do corpo, sem rosto)</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>dia-das-criancas_pulseira_lifestyle-com-tema</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
-Tema visual: Dia das Crianças. Paleta de cores: tons pastéis vibrantes (amarelo, azul-bebê, rosa-claro). Elementos/props de cena: pequenos balões desfocados ao fundo, ambiente lúdico. Clima geral: leve, alegre e descontraído.
-Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um pulso e uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou uma segunda mão aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I25" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J25" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K25" s="6" t="inlineStr"/>
-      <c r="L25" s="6" t="inlineStr"/>
-    </row>
-    <row r="26" ht="140" customHeight="1">
-      <c r="A26" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>Dia dos Pais</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
-        <is>
-          <t>Brinco</t>
-        </is>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>Still com Tema</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr"/>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>dia-dos-pais_brinco_still-com-tema</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
-Tema visual: Dia dos Pais. Paleta de cores: tons de azul-marinho e cinza-grafite. Elementos/props de cena: madeira escura, textura de couro ao fundo desfocado. Clima geral: sóbrio, elegante e masculino.
-Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I26" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J26" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K26" s="6" t="inlineStr"/>
-      <c r="L26" s="6" t="inlineStr"/>
-    </row>
-    <row r="27" ht="140" customHeight="1">
-      <c r="A27" s="6" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>Dia dos Pais</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>Brinco</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>Lifestyle com Tema</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>Sim (parte do corpo, sem rosto)</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>dia-dos-pais_brinco_lifestyle-com-tema</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
-Tema visual: Dia dos Pais. Paleta de cores: tons de azul-marinho e cinza-grafite. Elementos/props de cena: madeira escura, textura de couro ao fundo desfocado. Clima geral: sóbrio, elegante e masculino.
-Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto) — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Garanta anatomia perfeita da orelha e do lóbulo — sem deformações, sem uma segunda orelha ou rosto fantasma aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I27" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J27" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K27" s="6" t="inlineStr"/>
-      <c r="L27" s="6" t="inlineStr"/>
-    </row>
-    <row r="28" ht="140" customHeight="1">
-      <c r="A28" s="6" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>Dia dos Pais</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>Colar</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>Still com Tema</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr"/>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>dia-dos-pais_colar_still-com-tema</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
-Tema visual: Dia dos Pais. Paleta de cores: tons de azul-marinho e cinza-grafite. Elementos/props de cena: madeira escura, textura de couro ao fundo desfocado. Clima geral: sóbrio, elegante e masculino.
-Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I28" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J28" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K28" s="6" t="inlineStr"/>
-      <c r="L28" s="6" t="inlineStr"/>
-    </row>
-    <row r="29" ht="140" customHeight="1">
-      <c r="A29" s="6" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" s="6" t="inlineStr">
-        <is>
-          <t>Dia dos Pais</t>
-        </is>
-      </c>
-      <c r="C29" s="6" t="inlineStr">
-        <is>
-          <t>Colar</t>
-        </is>
-      </c>
-      <c r="D29" s="6" t="inlineStr">
-        <is>
-          <t>Lifestyle com Tema</t>
-        </is>
-      </c>
-      <c r="E29" s="6" t="inlineStr">
-        <is>
-          <t>Sim (parte do corpo, sem rosto)</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="inlineStr">
-        <is>
-          <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
-        </is>
-      </c>
-      <c r="G29" s="6" t="inlineStr">
-        <is>
-          <t>dia-dos-pais_colar_lifestyle-com-tema</t>
-        </is>
-      </c>
-      <c r="H29" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
-Tema visual: Dia dos Pais. Paleta de cores: tons de azul-marinho e cinza-grafite. Elementos/props de cena: madeira escura, textura de couro ao fundo desfocado. Clima geral: sóbrio, elegante e masculino.
-Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I29" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J29" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K29" s="6" t="inlineStr"/>
-      <c r="L29" s="6" t="inlineStr"/>
-    </row>
-    <row r="30" ht="140" customHeight="1">
-      <c r="A30" s="6" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t>Dia dos Pais</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
-          <t>Anel</t>
-        </is>
-      </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>Still com Tema</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="inlineStr"/>
-      <c r="G30" s="6" t="inlineStr">
-        <is>
-          <t>dia-dos-pais_anel_still-com-tema</t>
-        </is>
-      </c>
-      <c r="H30" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
-Tema visual: Dia dos Pais. Paleta de cores: tons de azul-marinho e cinza-grafite. Elementos/props de cena: madeira escura, textura de couro ao fundo desfocado. Clima geral: sóbrio, elegante e masculino.
-Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I30" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J30" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K30" s="6" t="inlineStr"/>
-      <c r="L30" s="6" t="inlineStr"/>
-    </row>
-    <row r="31" ht="140" customHeight="1">
-      <c r="A31" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" s="6" t="inlineStr">
-        <is>
-          <t>Dia dos Pais</t>
-        </is>
-      </c>
-      <c r="C31" s="6" t="inlineStr">
-        <is>
-          <t>Anel</t>
-        </is>
-      </c>
-      <c r="D31" s="6" t="inlineStr">
-        <is>
-          <t>Lifestyle com Tema</t>
-        </is>
-      </c>
-      <c r="E31" s="6" t="inlineStr">
-        <is>
-          <t>Sim (parte do corpo, sem rosto)</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="inlineStr">
-        <is>
-          <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>dia-dos-pais_anel_lifestyle-com-tema</t>
-        </is>
-      </c>
-      <c r="H31" s="6" t="inlineStr">
         <is>
           <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
@@ -5724,50 +5056,50 @@
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, dedos fundidos, articulações deformadas ou uma segunda mão/braço aparecendo parcialmente no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
-      <c r="I31" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J31" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K31" s="6" t="inlineStr"/>
-      <c r="L31" s="6" t="inlineStr"/>
-    </row>
-    <row r="32" ht="140" customHeight="1">
-      <c r="A32" s="6" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="J23" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="K23" s="6" t="inlineStr"/>
+      <c r="L23" s="6" t="inlineStr"/>
+    </row>
+    <row r="24" ht="140" customHeight="1">
+      <c r="A24" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>Dia dos Pais</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>Pulseira</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>Still com Tema</t>
         </is>
       </c>
-      <c r="E32" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="inlineStr"/>
-      <c r="G32" s="6" t="inlineStr">
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr"/>
+      <c r="G24" s="6" t="inlineStr">
         <is>
           <t>dia-dos-pais_pulseira_still-com-tema</t>
         </is>
       </c>
-      <c r="H32" s="6" t="inlineStr">
+      <c r="H24" s="6" t="inlineStr">
         <is>
           <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
@@ -5776,54 +5108,54 @@
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
-      <c r="I32" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J32" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K32" s="6" t="inlineStr"/>
-      <c r="L32" s="6" t="inlineStr"/>
-    </row>
-    <row r="33" ht="140" customHeight="1">
-      <c r="A33" s="6" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" s="6" t="inlineStr">
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="J24" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="K24" s="6" t="inlineStr"/>
+      <c r="L24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25" ht="140" customHeight="1">
+      <c r="A25" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>Dia dos Pais</t>
         </is>
       </c>
-      <c r="C33" s="6" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>Pulseira</t>
         </is>
       </c>
-      <c r="D33" s="6" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>Lifestyle com Tema</t>
         </is>
       </c>
-      <c r="E33" s="6" t="inlineStr">
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>Sim (parte do corpo, sem rosto)</t>
         </is>
       </c>
-      <c r="F33" s="6" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
         </is>
       </c>
-      <c r="G33" s="6" t="inlineStr">
+      <c r="G25" s="6" t="inlineStr">
         <is>
           <t>dia-dos-pais_pulseira_lifestyle-com-tema</t>
         </is>
       </c>
-      <c r="H33" s="6" t="inlineStr">
+      <c r="H25" s="6" t="inlineStr">
         <is>
           <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
@@ -5832,106 +5164,106 @@
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um pulso e uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou uma segunda mão aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
-      <c r="I33" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J33" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K33" s="6" t="inlineStr"/>
-      <c r="L33" s="6" t="inlineStr"/>
-    </row>
-    <row r="34" ht="140" customHeight="1">
-      <c r="A34" s="6" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" s="6" t="inlineStr">
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="J25" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="K25" s="6" t="inlineStr"/>
+      <c r="L25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26" ht="140" customHeight="1">
+      <c r="A26" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>Dia dos Pais</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>Brinco</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>Still com Tema</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr"/>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>dia-dos-pais_brinco_still-com-tema</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
+Tema visual: Dia dos Pais. Paleta de cores: tons de azul-marinho e cinza-grafite. Elementos/props de cena: madeira escura, textura de couro ao fundo desfocado. Clima geral: sóbrio, elegante e masculino.
+Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="J26" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="K26" s="6" t="inlineStr"/>
+      <c r="L26" s="6" t="inlineStr"/>
+    </row>
+    <row r="27" ht="140" customHeight="1">
+      <c r="A27" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>Dia Internacional da Mulher</t>
         </is>
       </c>
-      <c r="C34" s="6" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>Brinco</t>
         </is>
       </c>
-      <c r="D34" s="6" t="inlineStr">
-        <is>
-          <t>Still com Tema</t>
-        </is>
-      </c>
-      <c r="E34" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="inlineStr"/>
-      <c r="G34" s="6" t="inlineStr">
-        <is>
-          <t>dia-internacional-da-mulher_brinco_still-com-tema</t>
-        </is>
-      </c>
-      <c r="H34" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
-Tema visual: Dia Internacional da Mulher. Paleta de cores: tons de roxo e violeta. Elementos/props de cena: flor de mimosa (amarela) desfocada ao fundo. Clima geral: moderno, empoderado e sofisticado.
-Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I34" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J34" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K34" s="6" t="inlineStr"/>
-      <c r="L34" s="6" t="inlineStr"/>
-    </row>
-    <row r="35" ht="140" customHeight="1">
-      <c r="A35" s="6" t="n">
-        <v>34</v>
-      </c>
-      <c r="B35" s="6" t="inlineStr">
-        <is>
-          <t>Dia Internacional da Mulher</t>
-        </is>
-      </c>
-      <c r="C35" s="6" t="inlineStr">
-        <is>
-          <t>Brinco</t>
-        </is>
-      </c>
-      <c r="D35" s="6" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>Lifestyle com Tema</t>
         </is>
       </c>
-      <c r="E35" s="6" t="inlineStr">
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>Sim (parte do corpo, sem rosto)</t>
         </is>
       </c>
-      <c r="F35" s="6" t="inlineStr">
+      <c r="F27" s="6" t="inlineStr">
         <is>
           <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
         </is>
       </c>
-      <c r="G35" s="6" t="inlineStr">
+      <c r="G27" s="6" t="inlineStr">
         <is>
           <t>dia-internacional-da-mulher_brinco_lifestyle-com-tema</t>
         </is>
       </c>
-      <c r="H35" s="6" t="inlineStr">
+      <c r="H27" s="6" t="inlineStr">
         <is>
           <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
@@ -5940,50 +5272,50 @@
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Garanta anatomia perfeita da orelha e do lóbulo — sem deformações, sem uma segunda orelha ou rosto fantasma aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
-      <c r="I35" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J35" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K35" s="6" t="inlineStr"/>
-      <c r="L35" s="6" t="inlineStr"/>
-    </row>
-    <row r="36" ht="140" customHeight="1">
-      <c r="A36" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="B36" s="6" t="inlineStr">
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="J27" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="K27" s="6" t="inlineStr"/>
+      <c r="L27" s="6" t="inlineStr"/>
+    </row>
+    <row r="28" ht="140" customHeight="1">
+      <c r="A28" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>Dia Internacional da Mulher</t>
         </is>
       </c>
-      <c r="C36" s="6" t="inlineStr">
+      <c r="C28" s="6" t="inlineStr">
         <is>
           <t>Colar</t>
         </is>
       </c>
-      <c r="D36" s="6" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>Still com Tema</t>
         </is>
       </c>
-      <c r="E36" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="inlineStr"/>
-      <c r="G36" s="6" t="inlineStr">
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr"/>
+      <c r="G28" s="6" t="inlineStr">
         <is>
           <t>dia-internacional-da-mulher_colar_still-com-tema</t>
         </is>
       </c>
-      <c r="H36" s="6" t="inlineStr">
+      <c r="H28" s="6" t="inlineStr">
         <is>
           <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
@@ -5992,54 +5324,54 @@
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
-      <c r="I36" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J36" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K36" s="6" t="inlineStr"/>
-      <c r="L36" s="6" t="inlineStr"/>
-    </row>
-    <row r="37" ht="140" customHeight="1">
-      <c r="A37" s="6" t="n">
-        <v>36</v>
-      </c>
-      <c r="B37" s="6" t="inlineStr">
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="J28" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="K28" s="6" t="inlineStr"/>
+      <c r="L28" s="6" t="inlineStr"/>
+    </row>
+    <row r="29" ht="140" customHeight="1">
+      <c r="A29" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>Dia Internacional da Mulher</t>
         </is>
       </c>
-      <c r="C37" s="6" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>Colar</t>
         </is>
       </c>
-      <c r="D37" s="6" t="inlineStr">
+      <c r="D29" s="6" t="inlineStr">
         <is>
           <t>Lifestyle com Tema</t>
         </is>
       </c>
-      <c r="E37" s="6" t="inlineStr">
+      <c r="E29" s="6" t="inlineStr">
         <is>
           <t>Sim (parte do corpo, sem rosto)</t>
         </is>
       </c>
-      <c r="F37" s="6" t="inlineStr">
+      <c r="F29" s="6" t="inlineStr">
         <is>
           <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
         </is>
       </c>
-      <c r="G37" s="6" t="inlineStr">
+      <c r="G29" s="6" t="inlineStr">
         <is>
           <t>dia-internacional-da-mulher_colar_lifestyle-com-tema</t>
         </is>
       </c>
-      <c r="H37" s="6" t="inlineStr">
+      <c r="H29" s="6" t="inlineStr">
         <is>
           <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
@@ -6048,50 +5380,50 @@
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
-      <c r="I37" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J37" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K37" s="6" t="inlineStr"/>
-      <c r="L37" s="6" t="inlineStr"/>
-    </row>
-    <row r="38" ht="140" customHeight="1">
-      <c r="A38" s="6" t="n">
-        <v>37</v>
-      </c>
-      <c r="B38" s="6" t="inlineStr">
+      <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="J29" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="K29" s="6" t="inlineStr"/>
+      <c r="L29" s="6" t="inlineStr"/>
+    </row>
+    <row r="30" ht="140" customHeight="1">
+      <c r="A30" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>Dia Internacional da Mulher</t>
         </is>
       </c>
-      <c r="C38" s="6" t="inlineStr">
+      <c r="C30" s="6" t="inlineStr">
         <is>
           <t>Anel</t>
         </is>
       </c>
-      <c r="D38" s="6" t="inlineStr">
+      <c r="D30" s="6" t="inlineStr">
         <is>
           <t>Still com Tema</t>
         </is>
       </c>
-      <c r="E38" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F38" s="6" t="inlineStr"/>
-      <c r="G38" s="6" t="inlineStr">
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr"/>
+      <c r="G30" s="6" t="inlineStr">
         <is>
           <t>dia-internacional-da-mulher_anel_still-com-tema</t>
         </is>
       </c>
-      <c r="H38" s="6" t="inlineStr">
+      <c r="H30" s="6" t="inlineStr">
         <is>
           <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
@@ -6100,54 +5432,54 @@
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
-      <c r="I38" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J38" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K38" s="6" t="inlineStr"/>
-      <c r="L38" s="6" t="inlineStr"/>
-    </row>
-    <row r="39" ht="140" customHeight="1">
-      <c r="A39" s="6" t="n">
-        <v>38</v>
-      </c>
-      <c r="B39" s="6" t="inlineStr">
+      <c r="I30" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="J30" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="K30" s="6" t="inlineStr"/>
+      <c r="L30" s="6" t="inlineStr"/>
+    </row>
+    <row r="31" ht="140" customHeight="1">
+      <c r="A31" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>Dia Internacional da Mulher</t>
         </is>
       </c>
-      <c r="C39" s="6" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>Anel</t>
         </is>
       </c>
-      <c r="D39" s="6" t="inlineStr">
+      <c r="D31" s="6" t="inlineStr">
         <is>
           <t>Lifestyle com Tema</t>
         </is>
       </c>
-      <c r="E39" s="6" t="inlineStr">
+      <c r="E31" s="6" t="inlineStr">
         <is>
           <t>Sim (parte do corpo, sem rosto)</t>
         </is>
       </c>
-      <c r="F39" s="6" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
         <is>
           <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
         </is>
       </c>
-      <c r="G39" s="6" t="inlineStr">
+      <c r="G31" s="6" t="inlineStr">
         <is>
           <t>dia-internacional-da-mulher_anel_lifestyle-com-tema</t>
         </is>
       </c>
-      <c r="H39" s="6" t="inlineStr">
+      <c r="H31" s="6" t="inlineStr">
         <is>
           <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
@@ -6156,1022 +5488,158 @@
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, dedos fundidos, articulações deformadas ou uma segunda mão/braço aparecendo parcialmente no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
-      <c r="I39" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J39" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K39" s="6" t="inlineStr"/>
-      <c r="L39" s="6" t="inlineStr"/>
-    </row>
-    <row r="40" ht="140" customHeight="1">
-      <c r="A40" s="6" t="n">
-        <v>39</v>
-      </c>
-      <c r="B40" s="6" t="inlineStr">
-        <is>
-          <t>Dia Internacional da Mulher</t>
-        </is>
-      </c>
-      <c r="C40" s="6" t="inlineStr">
+      <c r="I31" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="J31" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="K31" s="6" t="inlineStr"/>
+      <c r="L31" s="6" t="inlineStr"/>
+    </row>
+    <row r="32" ht="140" customHeight="1">
+      <c r="A32" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Consciência Negra</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
         <is>
           <t>Pulseira</t>
         </is>
       </c>
-      <c r="D40" s="6" t="inlineStr">
+      <c r="D32" s="6" t="inlineStr">
         <is>
           <t>Still com Tema</t>
         </is>
       </c>
-      <c r="E40" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="inlineStr"/>
-      <c r="G40" s="6" t="inlineStr">
-        <is>
-          <t>dia-internacional-da-mulher_pulseira_still-com-tema</t>
-        </is>
-      </c>
-      <c r="H40" s="6" t="inlineStr">
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr"/>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>consciencia-negra_pulseira_still-com-tema</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
         <is>
           <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
-Tema visual: Dia Internacional da Mulher. Paleta de cores: tons de roxo e violeta. Elementos/props de cena: flor de mimosa (amarela) desfocada ao fundo. Clima geral: moderno, empoderado e sofisticado.
+Tema visual: Consciência Negra. Paleta de cores: tons terrosos e dourados. Elementos/props de cena: tecido com estampa de padronagem africana desfocado ao fundo. Clima geral: de valorização, orgulho e sofisticação.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
-      <c r="I40" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J40" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K40" s="6" t="inlineStr"/>
-      <c r="L40" s="6" t="inlineStr"/>
-    </row>
-    <row r="41" ht="140" customHeight="1">
-      <c r="A41" s="6" t="n">
-        <v>40</v>
-      </c>
-      <c r="B41" s="6" t="inlineStr">
-        <is>
-          <t>Dia Internacional da Mulher</t>
-        </is>
-      </c>
-      <c r="C41" s="6" t="inlineStr">
+      <c r="I32" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="J32" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="K32" s="6" t="inlineStr"/>
+      <c r="L32" s="6" t="inlineStr"/>
+    </row>
+    <row r="33" ht="140" customHeight="1">
+      <c r="A33" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>Consciência Negra</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>Pulseira</t>
         </is>
       </c>
-      <c r="D41" s="6" t="inlineStr">
+      <c r="D33" s="6" t="inlineStr">
         <is>
           <t>Lifestyle com Tema</t>
         </is>
       </c>
-      <c r="E41" s="6" t="inlineStr">
+      <c r="E33" s="6" t="inlineStr">
         <is>
           <t>Sim (parte do corpo, sem rosto)</t>
         </is>
       </c>
-      <c r="F41" s="6" t="inlineStr">
+      <c r="F33" s="6" t="inlineStr">
         <is>
           <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
         </is>
       </c>
-      <c r="G41" s="6" t="inlineStr">
-        <is>
-          <t>dia-internacional-da-mulher_pulseira_lifestyle-com-tema</t>
-        </is>
-      </c>
-      <c r="H41" s="6" t="inlineStr">
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>consciencia-negra_pulseira_lifestyle-com-tema</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="inlineStr">
         <is>
           <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
-Tema visual: Dia Internacional da Mulher. Paleta de cores: tons de roxo e violeta. Elementos/props de cena: flor de mimosa (amarela) desfocada ao fundo. Clima geral: moderno, empoderado e sofisticado.
+Tema visual: Consciência Negra. Paleta de cores: tons terrosos e dourados. Elementos/props de cena: tecido com estampa de padronagem africana desfocado ao fundo. Clima geral: de valorização, orgulho e sofisticação.
 Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um pulso e uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou uma segunda mão aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
-      <c r="I41" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J41" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K41" s="6" t="inlineStr"/>
-      <c r="L41" s="6" t="inlineStr"/>
-    </row>
-    <row r="42" ht="140" customHeight="1">
-      <c r="A42" s="6" t="n">
-        <v>41</v>
-      </c>
-      <c r="B42" s="6" t="inlineStr">
-        <is>
-          <t>Black Friday</t>
-        </is>
-      </c>
-      <c r="C42" s="6" t="inlineStr">
+      <c r="I33" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="J33" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="K33" s="6" t="inlineStr"/>
+      <c r="L33" s="6" t="inlineStr"/>
+    </row>
+    <row r="34" ht="140" customHeight="1">
+      <c r="A34" s="6" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>Consciência Negra</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
         <is>
           <t>Brinco</t>
         </is>
       </c>
-      <c r="D42" s="6" t="inlineStr">
+      <c r="D34" s="6" t="inlineStr">
         <is>
           <t>Still com Tema</t>
         </is>
       </c>
-      <c r="E42" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="inlineStr"/>
-      <c r="G42" s="6" t="inlineStr">
-        <is>
-          <t>black-friday_brinco_still-com-tema</t>
-        </is>
-      </c>
-      <c r="H42" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
-Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
-Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I42" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J42" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K42" s="6" t="inlineStr"/>
-      <c r="L42" s="6" t="inlineStr"/>
-    </row>
-    <row r="43" ht="140" customHeight="1">
-      <c r="A43" s="6" t="n">
-        <v>42</v>
-      </c>
-      <c r="B43" s="6" t="inlineStr">
-        <is>
-          <t>Black Friday</t>
-        </is>
-      </c>
-      <c r="C43" s="6" t="inlineStr">
-        <is>
-          <t>Brinco</t>
-        </is>
-      </c>
-      <c r="D43" s="6" t="inlineStr">
-        <is>
-          <t>Lifestyle com Tema</t>
-        </is>
-      </c>
-      <c r="E43" s="6" t="inlineStr">
-        <is>
-          <t>Sim (parte do corpo, sem rosto)</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="inlineStr">
-        <is>
-          <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
-        </is>
-      </c>
-      <c r="G43" s="6" t="inlineStr">
-        <is>
-          <t>black-friday_brinco_lifestyle-com-tema</t>
-        </is>
-      </c>
-      <c r="H43" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
-Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
-Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto) — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Garanta anatomia perfeita da orelha e do lóbulo — sem deformações, sem uma segunda orelha ou rosto fantasma aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I43" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J43" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K43" s="6" t="inlineStr"/>
-      <c r="L43" s="6" t="inlineStr"/>
-    </row>
-    <row r="44" ht="140" customHeight="1">
-      <c r="A44" s="6" t="n">
-        <v>43</v>
-      </c>
-      <c r="B44" s="6" t="inlineStr">
-        <is>
-          <t>Black Friday</t>
-        </is>
-      </c>
-      <c r="C44" s="6" t="inlineStr">
-        <is>
-          <t>Colar</t>
-        </is>
-      </c>
-      <c r="D44" s="6" t="inlineStr">
-        <is>
-          <t>Still com Tema</t>
-        </is>
-      </c>
-      <c r="E44" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="inlineStr"/>
-      <c r="G44" s="6" t="inlineStr">
-        <is>
-          <t>black-friday_colar_still-com-tema</t>
-        </is>
-      </c>
-      <c r="H44" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
-Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
-Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I44" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J44" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K44" s="6" t="inlineStr"/>
-      <c r="L44" s="6" t="inlineStr"/>
-    </row>
-    <row r="45" ht="140" customHeight="1">
-      <c r="A45" s="6" t="n">
-        <v>44</v>
-      </c>
-      <c r="B45" s="6" t="inlineStr">
-        <is>
-          <t>Black Friday</t>
-        </is>
-      </c>
-      <c r="C45" s="6" t="inlineStr">
-        <is>
-          <t>Colar</t>
-        </is>
-      </c>
-      <c r="D45" s="6" t="inlineStr">
-        <is>
-          <t>Lifestyle com Tema</t>
-        </is>
-      </c>
-      <c r="E45" s="6" t="inlineStr">
-        <is>
-          <t>Sim (parte do corpo, sem rosto)</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="inlineStr">
-        <is>
-          <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
-        </is>
-      </c>
-      <c r="G45" s="6" t="inlineStr">
-        <is>
-          <t>black-friday_colar_lifestyle-com-tema</t>
-        </is>
-      </c>
-      <c r="H45" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
-Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
-Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I45" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J45" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K45" s="6" t="inlineStr"/>
-      <c r="L45" s="6" t="inlineStr"/>
-    </row>
-    <row r="46" ht="140" customHeight="1">
-      <c r="A46" s="6" t="n">
-        <v>45</v>
-      </c>
-      <c r="B46" s="6" t="inlineStr">
-        <is>
-          <t>Black Friday</t>
-        </is>
-      </c>
-      <c r="C46" s="6" t="inlineStr">
-        <is>
-          <t>Anel</t>
-        </is>
-      </c>
-      <c r="D46" s="6" t="inlineStr">
-        <is>
-          <t>Still com Tema</t>
-        </is>
-      </c>
-      <c r="E46" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F46" s="6" t="inlineStr"/>
-      <c r="G46" s="6" t="inlineStr">
-        <is>
-          <t>black-friday_anel_still-com-tema</t>
-        </is>
-      </c>
-      <c r="H46" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
-Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
-Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I46" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J46" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K46" s="6" t="inlineStr"/>
-      <c r="L46" s="6" t="inlineStr"/>
-    </row>
-    <row r="47" ht="140" customHeight="1">
-      <c r="A47" s="6" t="n">
-        <v>46</v>
-      </c>
-      <c r="B47" s="6" t="inlineStr">
-        <is>
-          <t>Black Friday</t>
-        </is>
-      </c>
-      <c r="C47" s="6" t="inlineStr">
-        <is>
-          <t>Anel</t>
-        </is>
-      </c>
-      <c r="D47" s="6" t="inlineStr">
-        <is>
-          <t>Lifestyle com Tema</t>
-        </is>
-      </c>
-      <c r="E47" s="6" t="inlineStr">
-        <is>
-          <t>Sim (parte do corpo, sem rosto)</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="inlineStr">
-        <is>
-          <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
-        </is>
-      </c>
-      <c r="G47" s="6" t="inlineStr">
-        <is>
-          <t>black-friday_anel_lifestyle-com-tema</t>
-        </is>
-      </c>
-      <c r="H47" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
-Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
-Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a mão e os dedos — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, dedos fundidos, articulações deformadas ou uma segunda mão/braço aparecendo parcialmente no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I47" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J47" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K47" s="6" t="inlineStr"/>
-      <c r="L47" s="6" t="inlineStr"/>
-    </row>
-    <row r="48" ht="140" customHeight="1">
-      <c r="A48" s="6" t="n">
-        <v>47</v>
-      </c>
-      <c r="B48" s="6" t="inlineStr">
-        <is>
-          <t>Black Friday</t>
-        </is>
-      </c>
-      <c r="C48" s="6" t="inlineStr">
-        <is>
-          <t>Pulseira</t>
-        </is>
-      </c>
-      <c r="D48" s="6" t="inlineStr">
-        <is>
-          <t>Still com Tema</t>
-        </is>
-      </c>
-      <c r="E48" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F48" s="6" t="inlineStr"/>
-      <c r="G48" s="6" t="inlineStr">
-        <is>
-          <t>black-friday_pulseira_still-com-tema</t>
-        </is>
-      </c>
-      <c r="H48" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
-Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
-Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I48" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J48" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K48" s="6" t="inlineStr"/>
-      <c r="L48" s="6" t="inlineStr"/>
-    </row>
-    <row r="49" ht="140" customHeight="1">
-      <c r="A49" s="6" t="n">
-        <v>48</v>
-      </c>
-      <c r="B49" s="6" t="inlineStr">
-        <is>
-          <t>Black Friday</t>
-        </is>
-      </c>
-      <c r="C49" s="6" t="inlineStr">
-        <is>
-          <t>Pulseira</t>
-        </is>
-      </c>
-      <c r="D49" s="6" t="inlineStr">
-        <is>
-          <t>Lifestyle com Tema</t>
-        </is>
-      </c>
-      <c r="E49" s="6" t="inlineStr">
-        <is>
-          <t>Sim (parte do corpo, sem rosto)</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="inlineStr">
-        <is>
-          <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
-        </is>
-      </c>
-      <c r="G49" s="6" t="inlineStr">
-        <is>
-          <t>black-friday_pulseira_lifestyle-com-tema</t>
-        </is>
-      </c>
-      <c r="H49" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
-Tema visual: Black Friday. Paleta de cores: preto e dourado. Elementos/props de cena: fundo preto fosco, iluminação dramática lateral, reflexo dourado sutil. Clima geral: luxuoso, de destaque, alto contraste.
-Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um pulso e uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou uma segunda mão aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I49" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J49" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K49" s="6" t="inlineStr"/>
-      <c r="L49" s="6" t="inlineStr"/>
-    </row>
-    <row r="50" ht="140" customHeight="1">
-      <c r="A50" s="6" t="n">
-        <v>49</v>
-      </c>
-      <c r="B50" s="6" t="inlineStr">
-        <is>
-          <t>Natal</t>
-        </is>
-      </c>
-      <c r="C50" s="6" t="inlineStr">
-        <is>
-          <t>Brinco</t>
-        </is>
-      </c>
-      <c r="D50" s="6" t="inlineStr">
-        <is>
-          <t>Still com Tema</t>
-        </is>
-      </c>
-      <c r="E50" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="inlineStr"/>
-      <c r="G50" s="6" t="inlineStr">
-        <is>
-          <t>natal_brinco_still-com-tema</t>
-        </is>
-      </c>
-      <c r="H50" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
-Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
-Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I50" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J50" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K50" s="6" t="inlineStr"/>
-      <c r="L50" s="6" t="inlineStr"/>
-    </row>
-    <row r="51" ht="140" customHeight="1">
-      <c r="A51" s="6" t="n">
-        <v>50</v>
-      </c>
-      <c r="B51" s="6" t="inlineStr">
-        <is>
-          <t>Natal</t>
-        </is>
-      </c>
-      <c r="C51" s="6" t="inlineStr">
-        <is>
-          <t>Brinco</t>
-        </is>
-      </c>
-      <c r="D51" s="6" t="inlineStr">
-        <is>
-          <t>Lifestyle com Tema</t>
-        </is>
-      </c>
-      <c r="E51" s="6" t="inlineStr">
-        <is>
-          <t>Sim (parte do corpo, sem rosto)</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="inlineStr">
-        <is>
-          <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
-        </is>
-      </c>
-      <c r="G51" s="6" t="inlineStr">
-        <is>
-          <t>natal_brinco_lifestyle-com-tema</t>
-        </is>
-      </c>
-      <c r="H51" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
-Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
-Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto) — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Garanta anatomia perfeita da orelha e do lóbulo — sem deformações, sem uma segunda orelha ou rosto fantasma aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I51" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J51" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K51" s="6" t="inlineStr"/>
-      <c r="L51" s="6" t="inlineStr"/>
-    </row>
-    <row r="52" ht="140" customHeight="1">
-      <c r="A52" s="6" t="n">
-        <v>51</v>
-      </c>
-      <c r="B52" s="6" t="inlineStr">
-        <is>
-          <t>Natal</t>
-        </is>
-      </c>
-      <c r="C52" s="6" t="inlineStr">
-        <is>
-          <t>Colar</t>
-        </is>
-      </c>
-      <c r="D52" s="6" t="inlineStr">
-        <is>
-          <t>Still com Tema</t>
-        </is>
-      </c>
-      <c r="E52" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F52" s="6" t="inlineStr"/>
-      <c r="G52" s="6" t="inlineStr">
-        <is>
-          <t>natal_colar_still-com-tema</t>
-        </is>
-      </c>
-      <c r="H52" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
-Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
-Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I52" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J52" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K52" s="6" t="inlineStr"/>
-      <c r="L52" s="6" t="inlineStr"/>
-    </row>
-    <row r="53" ht="140" customHeight="1">
-      <c r="A53" s="6" t="n">
-        <v>52</v>
-      </c>
-      <c r="B53" s="6" t="inlineStr">
-        <is>
-          <t>Natal</t>
-        </is>
-      </c>
-      <c r="C53" s="6" t="inlineStr">
-        <is>
-          <t>Colar</t>
-        </is>
-      </c>
-      <c r="D53" s="6" t="inlineStr">
-        <is>
-          <t>Lifestyle com Tema</t>
-        </is>
-      </c>
-      <c r="E53" s="6" t="inlineStr">
-        <is>
-          <t>Sim (parte do corpo, sem rosto)</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="inlineStr">
-        <is>
-          <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
-        </is>
-      </c>
-      <c r="G53" s="6" t="inlineStr">
-        <is>
-          <t>natal_colar_lifestyle-com-tema</t>
-        </is>
-      </c>
-      <c r="H53" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
-Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
-Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I53" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J53" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K53" s="6" t="inlineStr"/>
-      <c r="L53" s="6" t="inlineStr"/>
-    </row>
-    <row r="54" ht="140" customHeight="1">
-      <c r="A54" s="6" t="n">
-        <v>53</v>
-      </c>
-      <c r="B54" s="6" t="inlineStr">
-        <is>
-          <t>Natal</t>
-        </is>
-      </c>
-      <c r="C54" s="6" t="inlineStr">
-        <is>
-          <t>Anel</t>
-        </is>
-      </c>
-      <c r="D54" s="6" t="inlineStr">
-        <is>
-          <t>Still com Tema</t>
-        </is>
-      </c>
-      <c r="E54" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F54" s="6" t="inlineStr"/>
-      <c r="G54" s="6" t="inlineStr">
-        <is>
-          <t>natal_anel_still-com-tema</t>
-        </is>
-      </c>
-      <c r="H54" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
-Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
-Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I54" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J54" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K54" s="6" t="inlineStr"/>
-      <c r="L54" s="6" t="inlineStr"/>
-    </row>
-    <row r="55" ht="140" customHeight="1">
-      <c r="A55" s="6" t="n">
-        <v>54</v>
-      </c>
-      <c r="B55" s="6" t="inlineStr">
-        <is>
-          <t>Natal</t>
-        </is>
-      </c>
-      <c r="C55" s="6" t="inlineStr">
-        <is>
-          <t>Anel</t>
-        </is>
-      </c>
-      <c r="D55" s="6" t="inlineStr">
-        <is>
-          <t>Lifestyle com Tema</t>
-        </is>
-      </c>
-      <c r="E55" s="6" t="inlineStr">
-        <is>
-          <t>Sim (parte do corpo, sem rosto)</t>
-        </is>
-      </c>
-      <c r="F55" s="6" t="inlineStr">
-        <is>
-          <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
-        </is>
-      </c>
-      <c r="G55" s="6" t="inlineStr">
-        <is>
-          <t>natal_anel_lifestyle-com-tema</t>
-        </is>
-      </c>
-      <c r="H55" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
-Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
-Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a mão e os dedos — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, dedos fundidos, articulações deformadas ou uma segunda mão/braço aparecendo parcialmente no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I55" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J55" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K55" s="6" t="inlineStr"/>
-      <c r="L55" s="6" t="inlineStr"/>
-    </row>
-    <row r="56" ht="140" customHeight="1">
-      <c r="A56" s="6" t="n">
-        <v>55</v>
-      </c>
-      <c r="B56" s="6" t="inlineStr">
-        <is>
-          <t>Natal</t>
-        </is>
-      </c>
-      <c r="C56" s="6" t="inlineStr">
-        <is>
-          <t>Pulseira</t>
-        </is>
-      </c>
-      <c r="D56" s="6" t="inlineStr">
-        <is>
-          <t>Still com Tema</t>
-        </is>
-      </c>
-      <c r="E56" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F56" s="6" t="inlineStr"/>
-      <c r="G56" s="6" t="inlineStr">
-        <is>
-          <t>natal_pulseira_still-com-tema</t>
-        </is>
-      </c>
-      <c r="H56" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
-Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
-Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I56" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J56" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K56" s="6" t="inlineStr"/>
-      <c r="L56" s="6" t="inlineStr"/>
-    </row>
-    <row r="57" ht="140" customHeight="1">
-      <c r="A57" s="6" t="n">
-        <v>56</v>
-      </c>
-      <c r="B57" s="6" t="inlineStr">
-        <is>
-          <t>Natal</t>
-        </is>
-      </c>
-      <c r="C57" s="6" t="inlineStr">
-        <is>
-          <t>Pulseira</t>
-        </is>
-      </c>
-      <c r="D57" s="6" t="inlineStr">
-        <is>
-          <t>Lifestyle com Tema</t>
-        </is>
-      </c>
-      <c r="E57" s="6" t="inlineStr">
-        <is>
-          <t>Sim (parte do corpo, sem rosto)</t>
-        </is>
-      </c>
-      <c r="F57" s="6" t="inlineStr">
-        <is>
-          <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
-        </is>
-      </c>
-      <c r="G57" s="6" t="inlineStr">
-        <is>
-          <t>natal_pulseira_lifestyle-com-tema</t>
-        </is>
-      </c>
-      <c r="H57" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
-Tema visual: Natal. Paleta de cores: tons de vermelho, dourado e verde. Elementos/props de cena: ramos verdes, pinha desfocada, luzes de natal desfocadas ao fundo (efeito bokeh dourado). Clima geral: aconchegante, festivo e brilhante.
-Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um pulso e uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou uma segunda mão aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I57" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J57" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K57" s="6" t="inlineStr"/>
-      <c r="L57" s="6" t="inlineStr"/>
-    </row>
-    <row r="58" ht="140" customHeight="1">
-      <c r="A58" s="6" t="n">
-        <v>57</v>
-      </c>
-      <c r="B58" s="6" t="inlineStr">
-        <is>
-          <t>Consciência Negra</t>
-        </is>
-      </c>
-      <c r="C58" s="6" t="inlineStr">
-        <is>
-          <t>Brinco</t>
-        </is>
-      </c>
-      <c r="D58" s="6" t="inlineStr">
-        <is>
-          <t>Still com Tema</t>
-        </is>
-      </c>
-      <c r="E58" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F58" s="6" t="inlineStr"/>
-      <c r="G58" s="6" t="inlineStr">
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr"/>
+      <c r="G34" s="6" t="inlineStr">
         <is>
           <t>consciencia-negra_brinco_still-com-tema</t>
         </is>
       </c>
-      <c r="H58" s="6" t="inlineStr">
+      <c r="H34" s="6" t="inlineStr">
         <is>
           <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Deixe um brinco apoiado em pé, em ângulo de aproximadamente 45° em relação à câmera, e o outro brinco deitado naturalmente sobre a superfície ao lado. Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco — nunca deixe a tarraxa solta ou separada da peça.
@@ -7180,54 +5648,54 @@
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
-      <c r="I58" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J58" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K58" s="6" t="inlineStr"/>
-      <c r="L58" s="6" t="inlineStr"/>
-    </row>
-    <row r="59" ht="140" customHeight="1">
-      <c r="A59" s="6" t="n">
-        <v>58</v>
-      </c>
-      <c r="B59" s="6" t="inlineStr">
+      <c r="I34" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="J34" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="K34" s="6" t="inlineStr"/>
+      <c r="L34" s="6" t="inlineStr"/>
+    </row>
+    <row r="35" ht="140" customHeight="1">
+      <c r="A35" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
         <is>
           <t>Consciência Negra</t>
         </is>
       </c>
-      <c r="C59" s="6" t="inlineStr">
+      <c r="C35" s="6" t="inlineStr">
         <is>
           <t>Brinco</t>
         </is>
       </c>
-      <c r="D59" s="6" t="inlineStr">
+      <c r="D35" s="6" t="inlineStr">
         <is>
           <t>Lifestyle com Tema</t>
         </is>
       </c>
-      <c r="E59" s="6" t="inlineStr">
+      <c r="E35" s="6" t="inlineStr">
         <is>
           <t>Sim (parte do corpo, sem rosto)</t>
         </is>
       </c>
-      <c r="F59" s="6" t="inlineStr">
+      <c r="F35" s="6" t="inlineStr">
         <is>
           <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
         </is>
       </c>
-      <c r="G59" s="6" t="inlineStr">
+      <c r="G35" s="6" t="inlineStr">
         <is>
           <t>consciencia-negra_brinco_lifestyle-com-tema</t>
         </is>
       </c>
-      <c r="H59" s="6" t="inlineStr">
+      <c r="H35" s="6" t="inlineStr">
         <is>
           <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: mostrar apenas a orelha e a lateral do rosto (apenas esses elementos — não mostrar o restante do rosto), evidenciando a peça de forma natural.
@@ -7236,50 +5704,50 @@
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Garanta anatomia perfeita da orelha e do lóbulo — sem deformações, sem uma segunda orelha ou rosto fantasma aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
-      <c r="I59" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J59" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K59" s="6" t="inlineStr"/>
-      <c r="L59" s="6" t="inlineStr"/>
-    </row>
-    <row r="60" ht="140" customHeight="1">
-      <c r="A60" s="6" t="n">
-        <v>59</v>
-      </c>
-      <c r="B60" s="6" t="inlineStr">
+      <c r="I35" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="J35" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="K35" s="6" t="inlineStr"/>
+      <c r="L35" s="6" t="inlineStr"/>
+    </row>
+    <row r="36" ht="140" customHeight="1">
+      <c r="A36" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>Consciência Negra</t>
         </is>
       </c>
-      <c r="C60" s="6" t="inlineStr">
+      <c r="C36" s="6" t="inlineStr">
         <is>
           <t>Colar</t>
         </is>
       </c>
-      <c r="D60" s="6" t="inlineStr">
+      <c r="D36" s="6" t="inlineStr">
         <is>
           <t>Still com Tema</t>
         </is>
       </c>
-      <c r="E60" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F60" s="6" t="inlineStr"/>
-      <c r="G60" s="6" t="inlineStr">
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr"/>
+      <c r="G36" s="6" t="inlineStr">
         <is>
           <t>consciencia-negra_colar_still-com-tema</t>
         </is>
       </c>
-      <c r="H60" s="6" t="inlineStr">
+      <c r="H36" s="6" t="inlineStr">
         <is>
           <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
 Composição: Apoie o colar completamente sobre a superfície, deixando a corrente cair em curvas amplas e orgânicas, como o peso natural do metal realmente se comportaria — nunca reproduza o formato exato da foto original. Nunca crie círculos perfeitos, ovais, corações, gotas ou curvas espelhadas/simétricas dos dois lados; cada lado da corrente deve ter um desenho diferente, com raios e comprimentos de curva variados. Se houver pingente, ele deve ser o ponto focal da composição.
@@ -7288,293 +5756,566 @@
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
-      <c r="I60" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J60" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K60" s="6" t="inlineStr"/>
-      <c r="L60" s="6" t="inlineStr"/>
-    </row>
-    <row r="61" ht="140" customHeight="1">
-      <c r="A61" s="6" t="n">
-        <v>60</v>
-      </c>
-      <c r="B61" s="6" t="inlineStr">
-        <is>
-          <t>Consciência Negra</t>
-        </is>
-      </c>
-      <c r="C61" s="6" t="inlineStr">
-        <is>
-          <t>Colar</t>
-        </is>
-      </c>
-      <c r="D61" s="6" t="inlineStr">
-        <is>
-          <t>Lifestyle com Tema</t>
-        </is>
-      </c>
-      <c r="E61" s="6" t="inlineStr">
-        <is>
-          <t>Sim (parte do corpo, sem rosto)</t>
-        </is>
-      </c>
-      <c r="F61" s="6" t="inlineStr">
-        <is>
-          <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
-        </is>
-      </c>
-      <c r="G61" s="6" t="inlineStr">
-        <is>
-          <t>consciencia-negra_colar_lifestyle-com-tema</t>
-        </is>
-      </c>
-      <c r="H61" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: mostrar apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula, evidenciando a peça de forma natural.
-Tema visual: Consciência Negra. Paleta de cores: tons terrosos e dourados. Elementos/props de cena: tecido com estampa de padronagem africana desfocado ao fundo. Clima geral: de valorização, orgulho e sofisticação.
-Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o colo, as clavículas e a parte inferior do pescoço, terminando imediatamente abaixo da mandíbula — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I61" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J61" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K61" s="6" t="inlineStr"/>
-      <c r="L61" s="6" t="inlineStr"/>
-    </row>
-    <row r="62" ht="140" customHeight="1">
-      <c r="A62" s="6" t="n">
-        <v>61</v>
-      </c>
-      <c r="B62" s="6" t="inlineStr">
-        <is>
-          <t>Consciência Negra</t>
-        </is>
-      </c>
-      <c r="C62" s="6" t="inlineStr">
-        <is>
-          <t>Anel</t>
-        </is>
-      </c>
-      <c r="D62" s="6" t="inlineStr">
-        <is>
-          <t>Still com Tema</t>
-        </is>
-      </c>
-      <c r="E62" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F62" s="6" t="inlineStr"/>
-      <c r="G62" s="6" t="inlineStr">
-        <is>
-          <t>consciencia-negra_anel_still-com-tema</t>
-        </is>
-      </c>
-      <c r="H62" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: Posicione o anel em pé, levemente inclinado, mostrando claramente o aro e o detalhe frontal (pedra ou desenho principal). A peça deve parecer fisicamente apoiada e equilibrada, nunca flutuando ou tombada.
-Tema visual: Consciência Negra. Paleta de cores: tons terrosos e dourados. Elementos/props de cena: tecido com estampa de padronagem africana desfocado ao fundo. Clima geral: de valorização, orgulho e sofisticação.
+      <c r="I36" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="J36" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="K36" s="6" t="inlineStr"/>
+      <c r="L36" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:L36"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Tipo de Peça</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Pose/Enquadramento</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Tem Modelo?</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Perfis Sugeridos</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Nome de Referência</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Prompt Mestre</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Proporção</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>Link da Imagem Gerada</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>Observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="130" customHeight="1">
+      <c r="A2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Expositor</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Expositor de Busto — Colar</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr"/>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>expositor_01_colar</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: Exiba a peça sobre um busto expositor feminino sem rosto, em resina fosca branca ou revestido em tecido linho cru, mostrando apenas a região do pescoço e dos ombros do busto (não mostrar a base nem o suporte inteiro). O colar deve cair naturalmente pela gravidade sobre a curva do busto, sem parecer colado ou flutuando.
+Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="inlineStr"/>
+      <c r="K2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3" ht="130" customHeight="1">
+      <c r="A3" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Expositor</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Expositor de Busto — Colar Longo</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr"/>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>expositor_02_colar-longo</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: Exiba a peça sobre um busto expositor feminino sem rosto, em resina fosca off-white, enquadrado da base do pescoço até o meio do tórax. A corrente deve descer naturalmente acompanhando o volume do busto, sem parecer colada ou desenhada.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
-      <c r="I62" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J62" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K62" s="6" t="inlineStr"/>
-      <c r="L62" s="6" t="inlineStr"/>
-    </row>
-    <row r="63" ht="140" customHeight="1">
-      <c r="A63" s="6" t="n">
-        <v>62</v>
-      </c>
-      <c r="B63" s="6" t="inlineStr">
-        <is>
-          <t>Consciência Negra</t>
-        </is>
-      </c>
-      <c r="C63" s="6" t="inlineStr">
-        <is>
-          <t>Anel</t>
-        </is>
-      </c>
-      <c r="D63" s="6" t="inlineStr">
-        <is>
-          <t>Lifestyle com Tema</t>
-        </is>
-      </c>
-      <c r="E63" s="6" t="inlineStr">
-        <is>
-          <t>Sim (parte do corpo, sem rosto)</t>
-        </is>
-      </c>
-      <c r="F63" s="6" t="inlineStr">
-        <is>
-          <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
-        </is>
-      </c>
-      <c r="G63" s="6" t="inlineStr">
-        <is>
-          <t>consciencia-negra_anel_lifestyle-com-tema</t>
-        </is>
-      </c>
-      <c r="H63" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: mostrar apenas a mão e os dedos, evidenciando a peça de forma natural.
-Tema visual: Consciência Negra. Paleta de cores: tons terrosos e dourados. Elementos/props de cena: tecido com estampa de padronagem africana desfocado ao fundo. Clima geral: de valorização, orgulho e sofisticação.
-Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas a mão e os dedos — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, dedos fundidos, articulações deformadas ou uma segunda mão/braço aparecendo parcialmente no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I63" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J63" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K63" s="6" t="inlineStr"/>
-      <c r="L63" s="6" t="inlineStr"/>
-    </row>
-    <row r="64" ht="140" customHeight="1">
-      <c r="A64" s="6" t="n">
-        <v>63</v>
-      </c>
-      <c r="B64" s="6" t="inlineStr">
-        <is>
-          <t>Consciência Negra</t>
-        </is>
-      </c>
-      <c r="C64" s="6" t="inlineStr">
-        <is>
-          <t>Pulseira</t>
-        </is>
-      </c>
-      <c r="D64" s="6" t="inlineStr">
-        <is>
-          <t>Still com Tema</t>
-        </is>
-      </c>
-      <c r="E64" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F64" s="6" t="inlineStr"/>
-      <c r="G64" s="6" t="inlineStr">
-        <is>
-          <t>consciencia-negra_pulseira_still-com-tema</t>
-        </is>
-      </c>
-      <c r="H64" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: Apoie a pulseira formando uma curva aberta e natural sobre a superfície, como se tivesse caído naturalmente — nunca um círculo perfeitamente fechado.
-Tema visual: Consciência Negra. Paleta de cores: tons terrosos e dourados. Elementos/props de cena: tecido com estampa de padronagem africana desfocado ao fundo. Clima geral: de valorização, orgulho e sofisticação.
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr"/>
+      <c r="K3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4" ht="130" customHeight="1">
+      <c r="A4" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Expositor</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Expositor de Mão — Anel</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr"/>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>expositor_03_anel</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: Exiba a peça em um suporte de mão expositor, em cerâmica ou resina fosca branca, com os dedos levemente afastados e curvatura anatômica realista — mostrar apenas a mão do expositor, sem pulso ou braço além do necessário.
+Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr"/>
+      <c r="K4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5" ht="130" customHeight="1">
+      <c r="A5" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Expositor</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Expositor de Mão — Pulseira/Bracelete</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr"/>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>expositor_04_pulseira</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: Exiba a peça em um suporte de pulso expositor cilíndrico, em madeira clara ou resina fosca, mostrando apenas o segmento do pulso — sem mão, dedos ou antebraço completo.
+Fotografia still editorial sobre uma superfície de mármore branco, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr"/>
+      <c r="K5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6" ht="130" customHeight="1">
+      <c r="A6" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Expositor</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Expositor de Orelha — Brinco</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr"/>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>expositor_05_brinco</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: Exiba o par de brincos em um suporte expositor no formato de orelha, em resina fosca branca ou acrílico transparente, mostrando apenas a peça do expositor (sem rosto ou cabeça). Caso a peça tenha tarraxa, mantenha uma tarraxa presa em cada brinco.
+Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr"/>
+      <c r="K6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7" ht="130" customHeight="1">
+      <c r="A7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Expositor</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Expositor de Orelha — Brinco (Cenário)</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr"/>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>expositor_06_brinco</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: Exiba o par de brincos em um suporte expositor no formato de orelha, em cerâmica fosca bege claro, sobre um pano acetinado off-white com dobras suaves ao fundo.
 Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
 Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
         </is>
       </c>
-      <c r="I64" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J64" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K64" s="6" t="inlineStr"/>
-      <c r="L64" s="6" t="inlineStr"/>
-    </row>
-    <row r="65" ht="140" customHeight="1">
-      <c r="A65" s="6" t="n">
-        <v>64</v>
-      </c>
-      <c r="B65" s="6" t="inlineStr">
-        <is>
-          <t>Consciência Negra</t>
-        </is>
-      </c>
-      <c r="C65" s="6" t="inlineStr">
-        <is>
-          <t>Pulseira</t>
-        </is>
-      </c>
-      <c r="D65" s="6" t="inlineStr">
-        <is>
-          <t>Lifestyle com Tema</t>
-        </is>
-      </c>
-      <c r="E65" s="6" t="inlineStr">
-        <is>
-          <t>Sim (parte do corpo, sem rosto)</t>
-        </is>
-      </c>
-      <c r="F65" s="6" t="inlineStr">
-        <is>
-          <t>Mulher jovem (18-25), pele clara | Mulher adulta (30-45), pele morena | Mulher adulta (30-45), pele negra | Mulher idosa (60+), pele clara</t>
-        </is>
-      </c>
-      <c r="G65" s="6" t="inlineStr">
-        <is>
-          <t>consciencia-negra_pulseira_lifestyle-com-tema</t>
-        </is>
-      </c>
-      <c r="H65" s="6" t="inlineStr">
-        <is>
-          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
-Composição: mostrar apenas o pulso, evidenciando a peça de forma natural.
-Tema visual: Consciência Negra. Paleta de cores: tons terrosos e dourados. Elementos/props de cena: tecido com estampa de padronagem africana desfocado ao fundo. Clima geral: de valorização, orgulho e sofisticação.
-Fotografia editorial extremamente realista para catálogo premium de joias, produzida como uma campanha de joalheria de luxo. Enquadramento fechado, mostrando apenas o pulso — nunca mostrar rosto, olhos, boca, nariz, cabelo ou outras partes do corpo além das indicadas. A pele deve ter aparência extremamente natural, saudável e uniforme, com tom: [PERFIL]. Criar uma única faixa de sombra diagonal, contínua e bem definida, inclinada aproximadamente 45°, atravessando a composição como luz entrando por uma janela — a sombra nunca deve cruzar ou escurecer a peça, que deve permanecer completamente iluminada e em destaque. Vestuário minimalista em tecido acetinado ou seda fosca, em tom off-white, extremamente discreto para não competir com a joia. Lente equivalente entre 85mm e 105mm, profundidade de campo rasa — a pele pode ficar levemente desfocada, mas a peça deve permanecer perfeitamente nítida. Fundo neutro (cinza quente muito suave ou bege acinzentado), sem textura, objetos ou elementos decorativos. Não adicionar outras joias, acessórios ou maquiagem chamativa.
-Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Mostre exatamente um pulso e uma mão, com exatamente cinco dedos anatomicamente corretos — nunca dedos extras, fundidos ou uma segunda mão aparecendo no enquadramento. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
-        </is>
-      </c>
-      <c r="I65" s="6" t="inlineStr">
-        <is>
-          <t>3:4 (vertical)</t>
-        </is>
-      </c>
-      <c r="J65" s="6" t="inlineStr">
-        <is>
-          <t>A gerar</t>
-        </is>
-      </c>
-      <c r="K65" s="6" t="inlineStr"/>
-      <c r="L65" s="6" t="inlineStr"/>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr"/>
+      <c r="K7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8" ht="130" customHeight="1">
+      <c r="A8" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Expositor</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Expositor de Correntes — Corrente Masculina</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr"/>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>expositor_07_corrente-masculina</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: Exiba a peça em um suporte expositor de correntes tipo T (cabideiro de mesa), em madeira escura ou metal fosco preto, mostrando apenas a barra horizontal do suporte — sem a base inteira. A corrente deve cair naturalmente dos dois lados da barra, formando curvas assimétricas.
+Fotografia still editorial sobre uma superfície de madeira clara, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr"/>
+      <c r="K8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9" ht="130" customHeight="1">
+      <c r="A9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Expositor</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Expositor de Correntes — Colar com Pingente</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr"/>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>expositor_08_pingente</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: Exiba a peça pendurada em um suporte expositor de correntes tipo T, em acrílico transparente ou resina fosca branca, com o pingente centralizado e voltado de frente para a câmera.
+Fotografia still de produto (packshot) profissional para e-commerce. Fundo branco puro (RGB 255,255,255), infinito, sem linha de horizonte, sem gradientes, sem textura e sem qualquer elemento decorativo. Iluminação de estúdio: uma fonte de luz principal ampla e difusa, uma luz de preenchimento suave do lado oposto para controlar sombras, e uma luz de contorno sutil para destacar a silhueta. Reflexos no metal limpos, contínuos e fisicamente corretos, sem brilhos estourados. Sombra de contato única, suave e difusa, com leve gradiente natural logo abaixo da peça. Lente equivalente entre 85mm e 105mm, foco perfeitamente nítido em toda a peça, sem distorção de perspectiva.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="inlineStr"/>
+      <c r="K9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10" ht="130" customHeight="1">
+      <c r="A10" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Expositor</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Expositor de Pescoço — Choker/Gargantilha</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr"/>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>expositor_09_choker-gargantilha</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: Exiba a peça em um suporte expositor cilíndrico de pescoço, em veludo fosco cinza-claro ou resina branca, mostrando apenas o cilindro — sem base larga ou pedestal completo.
+Fotografia still editorial sobre uma superfície de pedra calcária clara, de formato orgânico e bordas irregulares, apoiada sobre um tecido acetinado em tom bege claro e quente. Câmera em perspectiva oblíqua, entre 45° e 55° acima da superfície — nunca totalmente frontal nem top-down perfeitamente perpendicular; a composição pode aparecer levemente rotacionada dentro do quadro. Iluminação profissional de estúdio inspirada em luz solar suave entrando lateralmente, criando sombras pequenas e realistas que mostram a peça fisicamente apoiada sobre a superfície. Contraste moderado, cena clara, quente e sofisticada — evitar sombras muito escuras ou iluminação dramática.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr"/>
+      <c r="K10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11" ht="130" customHeight="1">
+      <c r="A11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Expositor</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Expositor Múltiplo — Conjunto</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr"/>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>expositor_10_conjunto-colar-+-brinco</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: Exiba as peças do conjunto distribuídas entre um busto expositor (colar) e um pequeno suporte de orelha ao lado (brincos), ambos em resina fosca da mesma tonalidade off-white, criando um display coordenado de vitrine — utilize exatamente as peças presentes na foto anexada, na mesma quantidade, sem adicionar ou remover nenhuma joia.
+Fotografia editorial de joias com estética minimalista, sofisticada e contemporânea, semelhante a campanhas de marcas de luxo. A peça deve estar apoiada sobre um tecido branco ou off-white premium, fosco, encorpado, com textura delicada semelhante a crepe de seda estruturado, moldado à mão em ondas amplas e curvas orgânicas — nunca padrões repetitivos, simetria perfeita ou dobras geométricas/espirais matematicamente exatas (isso denuncia aparência de imagem gerada por IA). Câmera em ângulo de aproximadamente 45°, lente macro equivalente a 85-100mm, enquadramento em close-up com a peça ocupando cerca da metade da imagem. Iluminação natural extremamente suave e difusa, como luz de uma grande janela lateral, criando sombras delicadas entre as dobras do tecido. Paleta restrita a branco quente, marfim e creme suave. Não adicionar flores, folhas, pedras decorativas, madeira, embalagens, mãos, pessoas ou qualquer elemento decorativo.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr"/>
+      <c r="K11" s="6" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L65"/>
+  <autoFilter ref="A1:K11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Adiciona categorias Lifestyle e Peças em Você ao catálogo
Lifestyle: 10 fotos com modelo genérica de rosto completo (5 mulheres
variando etnia, 5 homens), em cenas do dia a dia, seguindo o mesmo
mecanismo de uma foto anexada (a joia).

Peças em Você: 10 fotos que usam DUAS fotos anexadas — o rosto da
própria assinante + a foto da joia — preservando a identidade da
assinante e usando exclusivamente as joias da segunda foto. UI atualizada
com aviso de "anexe 2 fotos" no catálogo e instruções específicas na
página de prompt.

Também corrige a view "Todos os tipos" do catálogo para trazer as
seções de Datas Comemorativas abertas junto com o evergreen, em vez de
exigir a aba separada.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0184vv6VXBstbMukBGTFNCKP
</commit_message>
<xml_diff>
--- a/content/Photo_Studio_TPV_Biblioteca_de_Prompts.xlsx
+++ b/content/Photo_Studio_TPV_Biblioteca_de_Prompts.xlsx
@@ -11,11 +11,15 @@
     <sheet name="Evergreen" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Datas Comemorativas" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Expositores" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Lifestyle" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Peças em Você" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Evergreen'!$A$1:$K$66</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Datas Comemorativas'!$A$1:$L$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Expositores'!$A$1:$K$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Lifestyle'!$A$1:$K$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Peças em Você'!$A$1:$K$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -6318,4 +6322,1084 @@
   <autoFilter ref="A1:K11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Tipo de Peça</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Pose/Enquadramento</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Tem Modelo?</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Perfis Sugeridos</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Nome de Referência</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Prompt Mestre</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Proporção</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>Link da Imagem Gerada</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>Observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="130" customHeight="1">
+      <c r="A2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Mulher — Colar (Terraço)</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>Sim (rosto completo)</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr"/>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>lifestyle_01_mulher</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: Mulher negra, aproximadamente 30 anos, cabelo cacheado natural com volume, pele com brilho saudável. Ela está sentada em um terraço ensolarado, apoiada em uma mesa de vime clara, segurando uma xícara de café com as duas mãos próximas ao colo, sorrindo de forma leve e genuína enquanto olha para o horizonte, fora da câmera. Veste uma blusa de linho branca de gola V. Luz natural da manhã, suave e dourada, incidindo lateralmente. Enquadramento da cintura para cima, evidenciando pescoço e colo para valorizar o colar.
+Fotografia lifestyle hiper-realista para campanha de joias, em formato vertical 3:4 e altíssima resolução. Rosto e expressão da modelo aparecem naturalmente, sem pose rígida ou artificial — a cena deve parecer um flagrante espontâneo do dia a dia, nunca uma fotografia de estúdio posada. Lente equivalente a 85mm, profundidade de campo rasa, fundo suavemente desfocado. A joia permanece perfeitamente nítida e prioritária no foco, com reflexos fisicamente corretos no metal. Pele com textura natural, sem efeito plástico ou de filtro. Mãos, quando aparecerem, devem ter anatomia perfeita — sempre cinco dedos, nunca deformados, duplicados ou fundidos.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="inlineStr"/>
+      <c r="K2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3" ht="130" customHeight="1">
+      <c r="A3" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Mulher — Brinco e Anel (Café de Rua)</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Sim (rosto completo)</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr"/>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>lifestyle_02_mulher</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: Mulher branca, cabelo loiro liso preso em um rabo de cavalo baixo, sentada em uma mesinha de um café de rua em uma cidade europeia, apoiando o queixo em uma das mãos enquanto segura um pequeno espresso com a outra. Sorriso discreto, olhar para o lado, fora da câmera. Veste um blazer bege sobre uma blusa branca. Luz natural de fim de manhã, fria e nublada, sombras suaves. Enquadramento da cintura para cima, valorizando a orelha e a mão que segura o queixo.
+Fotografia lifestyle hiper-realista para campanha de joias, em formato vertical 3:4 e altíssima resolução. Rosto e expressão da modelo aparecem naturalmente, sem pose rígida ou artificial — a cena deve parecer um flagrante espontâneo do dia a dia, nunca uma fotografia de estúdio posada. Lente equivalente a 85mm, profundidade de campo rasa, fundo suavemente desfocado. A joia permanece perfeitamente nítida e prioritária no foco, com reflexos fisicamente corretos no metal. Pele com textura natural, sem efeito plástico ou de filtro. Mãos, quando aparecerem, devem ter anatomia perfeita — sempre cinco dedos, nunca deformados, duplicados ou fundidos.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr"/>
+      <c r="K3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4" ht="130" customHeight="1">
+      <c r="A4" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Mulher — Colar Longo (Janela)</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Sim (rosto completo)</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr"/>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>lifestyle_03_mulher</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: Mulher ruiva, cabelo ondulado solto sobre os ombros, em pé ao lado de uma grande janela com cortina translúcida, uma mão ajeitando delicadamente uma mecha de cabelo atrás da orelha enquanto olha para fora, expressão tranquila. Veste uma camisa de seda off-white. Luz natural lateral entrando pela janela, criando contraste suave entre luz e sombra no rosto. Enquadramento do peito para cima, evidenciando pescoço, colo e orelha.
+Fotografia lifestyle hiper-realista para campanha de joias, em formato vertical 3:4 e altíssima resolução. Rosto e expressão da modelo aparecem naturalmente, sem pose rígida ou artificial — a cena deve parecer um flagrante espontâneo do dia a dia, nunca uma fotografia de estúdio posada. Lente equivalente a 85mm, profundidade de campo rasa, fundo suavemente desfocado. A joia permanece perfeitamente nítida e prioritária no foco, com reflexos fisicamente corretos no metal. Pele com textura natural, sem efeito plástico ou de filtro. Mãos, quando aparecerem, devem ter anatomia perfeita — sempre cinco dedos, nunca deformados, duplicados ou fundidos.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr"/>
+      <c r="K4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5" ht="130" customHeight="1">
+      <c r="A5" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Mulher — Brinco (Jardim)</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Sim (rosto completo)</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr"/>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>lifestyle_04_mulher</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: Mulher negra de pele clara, cabelo trançado preso para trás, caminhando em um jardim com vegetação desfocada ao fundo, com a cabeça levemente inclinada para trás enquanto sorri abertamente para o céu, em um gesto espontâneo de alegria. Veste um vestido de linho verde-oliva sem mangas. Luz natural de tarde, quente, levemente contraluz. Enquadramento da cintura para cima, valorizando pescoço e orelhas.
+Fotografia lifestyle hiper-realista para campanha de joias, em formato vertical 3:4 e altíssima resolução. Rosto e expressão da modelo aparecem naturalmente, sem pose rígida ou artificial — a cena deve parecer um flagrante espontâneo do dia a dia, nunca uma fotografia de estúdio posada. Lente equivalente a 85mm, profundidade de campo rasa, fundo suavemente desfocado. A joia permanece perfeitamente nítida e prioritária no foco, com reflexos fisicamente corretos no metal. Pele com textura natural, sem efeito plástico ou de filtro. Mãos, quando aparecerem, devem ter anatomia perfeita — sempre cinco dedos, nunca deformados, duplicados ou fundidos.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr"/>
+      <c r="K5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6" ht="130" customHeight="1">
+      <c r="A6" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Mulher — Pulseira (Sofá)</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Sim (rosto completo)</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr"/>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>lifestyle_05_mulher</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: Mulher branca, cabelo castanho-claro solto com ondas suaves, sentada em um sofá bege em ambiente doméstico aconchegante, com uma das pernas dobrada sobre o assento, segurando um celular com as duas mãos e olhando para a tela com expressão tranquila. Veste uma camisa branca oversized. Luz natural suave de janela lateral, ambiente claro e minimalista. Enquadramento evidenciando mãos, pulsos e colo.
+Fotografia lifestyle hiper-realista para campanha de joias, em formato vertical 3:4 e altíssima resolução. Rosto e expressão da modelo aparecem naturalmente, sem pose rígida ou artificial — a cena deve parecer um flagrante espontâneo do dia a dia, nunca uma fotografia de estúdio posada. Lente equivalente a 85mm, profundidade de campo rasa, fundo suavemente desfocado. A joia permanece perfeitamente nítida e prioritária no foco, com reflexos fisicamente corretos no metal. Pele com textura natural, sem efeito plástico ou de filtro. Mãos, quando aparecerem, devem ter anatomia perfeita — sempre cinco dedos, nunca deformados, duplicados ou fundidos.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr"/>
+      <c r="K6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7" ht="130" customHeight="1">
+      <c r="A7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Homem — Corrente (Escritório)</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Sim (rosto completo)</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr"/>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>lifestyle_06_homem</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: Homem branco, aproximadamente 35 anos, cabelo curto bem cuidado, em pé junto a uma janela de um escritório moderno, uma mão no bolso da calça enquanto observa a paisagem urbana desfocada ao fundo, expressão séria e confiante. Veste uma camisa social azul-marinho com as mangas dobradas até o antebraço. Luz natural fria entrando pela janela, contraste moderado. Enquadramento do peito para cima, valorizando pescoço e punho.
+Fotografia lifestyle hiper-realista para campanha de joias, em formato vertical 3:4 e altíssima resolução. Rosto e expressão da modelo aparecem naturalmente, sem pose rígida ou artificial — a cena deve parecer um flagrante espontâneo do dia a dia, nunca uma fotografia de estúdio posada. Lente equivalente a 85mm, profundidade de campo rasa, fundo suavemente desfocado. A joia permanece perfeitamente nítida e prioritária no foco, com reflexos fisicamente corretos no metal. Pele com textura natural, sem efeito plástico ou de filtro. Mãos, quando aparecerem, devem ter anatomia perfeita — sempre cinco dedos, nunca deformados, duplicados ou fundidos.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr"/>
+      <c r="K7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8" ht="130" customHeight="1">
+      <c r="A8" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Homem — Pulseira (Rua)</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Sim (rosto completo)</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr"/>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>lifestyle_07_homem</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: Homem negro, cabelo curto raspado nas laterais, caminhando em uma rua urbana com paredes de tijolo desfocadas ao fundo, mãos nos bolsos de uma jaqueta jeans, olhar confiante direcionado para o lado, fora da câmera. Veste uma camiseta branca básica sob a jaqueta. Luz natural de fim de tarde, dourada e lateral. Enquadramento da cintura para cima, valorizando pulso e antebraço.
+Fotografia lifestyle hiper-realista para campanha de joias, em formato vertical 3:4 e altíssima resolução. Rosto e expressão da modelo aparecem naturalmente, sem pose rígida ou artificial — a cena deve parecer um flagrante espontâneo do dia a dia, nunca uma fotografia de estúdio posada. Lente equivalente a 85mm, profundidade de campo rasa, fundo suavemente desfocado. A joia permanece perfeitamente nítida e prioritária no foco, com reflexos fisicamente corretos no metal. Pele com textura natural, sem efeito plástico ou de filtro. Mãos, quando aparecerem, devem ter anatomia perfeita — sempre cinco dedos, nunca deformados, duplicados ou fundidos.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr"/>
+      <c r="K8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9" ht="130" customHeight="1">
+      <c r="A9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Homem — Anel (Café)</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Sim (rosto completo)</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr"/>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>lifestyle_08_homem</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: Homem branco com barba curta bem aparada, sentado em uma mesa de madeira em um café, segurando uma xícara de café preta com uma das mãos apoiada sobre a mesa, olhando para baixo em direção à xícara com expressão relaxada. Veste um suéter cinza de gola redonda. Luz natural suave de janela, tons quentes. Enquadramento fechado na mão e no antebraço apoiados sobre a mesa.
+Fotografia lifestyle hiper-realista para campanha de joias, em formato vertical 3:4 e altíssima resolução. Rosto e expressão da modelo aparecem naturalmente, sem pose rígida ou artificial — a cena deve parecer um flagrante espontâneo do dia a dia, nunca uma fotografia de estúdio posada. Lente equivalente a 85mm, profundidade de campo rasa, fundo suavemente desfocado. A joia permanece perfeitamente nítida e prioritária no foco, com reflexos fisicamente corretos no metal. Pele com textura natural, sem efeito plástico ou de filtro. Mãos, quando aparecerem, devem ter anatomia perfeita — sempre cinco dedos, nunca deformados, duplicados ou fundidos.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="inlineStr"/>
+      <c r="K9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10" ht="130" customHeight="1">
+      <c r="A10" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Homem — Corrente (Varanda)</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Sim (rosto completo)</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr"/>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>lifestyle_09_homem</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: Homem negro, cabelo curto, em pé em uma varanda ao entardecer, apoiado no parapeito com os dois antebraços, camisa social branca com os primeiros botões abertos, olhando para o horizonte com expressão tranquila. Luz dourada de fim de tarde, contraluz suave. Enquadramento do peito para cima, evidenciando pescoço e colo aberto pela camisa.
+Fotografia lifestyle hiper-realista para campanha de joias, em formato vertical 3:4 e altíssima resolução. Rosto e expressão da modelo aparecem naturalmente, sem pose rígida ou artificial — a cena deve parecer um flagrante espontâneo do dia a dia, nunca uma fotografia de estúdio posada. Lente equivalente a 85mm, profundidade de campo rasa, fundo suavemente desfocado. A joia permanece perfeitamente nítida e prioritária no foco, com reflexos fisicamente corretos no metal. Pele com textura natural, sem efeito plástico ou de filtro. Mãos, quando aparecerem, devem ter anatomia perfeita — sempre cinco dedos, nunca deformados, duplicados ou fundidos.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr"/>
+      <c r="K10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11" ht="130" customHeight="1">
+      <c r="A11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Homem — Pulseira (Externo)</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Sim (rosto completo)</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr"/>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>lifestyle_10_homem</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Utilize exclusivamente a joia da fotografia anexada como referência do produto. Antes de gerar, identifique exatamente quantas peças e quantas unidades de cada peça existem na fotografia anexada (por exemplo, um par de brincos conta como duas unidades) e reproduza exatamente essa mesma quantidade na imagem final — nunca invente, duplique, repita, clone, remova ou complete o conjunto adicionando peças, pingentes, pedras ou componentes que não estejam fisicamente presentes na foto original. Se a foto anexada não contiver determinado tipo de peça (por exemplo, não houver anel), essa peça não deve aparecer na imagem final sob nenhuma hipótese. Preserve com fidelidade absoluta: formato, proporções, espessura, acabamento, brilho, textura, cor do metal, pedras (corte, tamanho e posição), cravação, fechos e elos, e todos os demais detalhes originais da peça. Não redesenhe, reinterprete, estilize, complete, corrija ou invente nenhuma característica da joia — reproduza exatamente o que existe na imagem original. Não utilize a foto anexada como referência de cenário, iluminação, enquadramento ou composição — ela serve apenas para identificar a peça, sua quantidade exata e seus detalhes exatos; remova completamente quaisquer objetos, mãos ou fundos presentes na foto original. Atenção especial à espessura de correntes, elos e fios: é um erro comum de IA generativa deixar correntes finas e delicadas mais grossas, mais vistosas ou mais robustas do que a peça real. A corrente gerada precisa ter exatamente a mesma espessura, o mesmo diâmetro de elo e a mesma delicadeza da foto original — NUNCA mais grossa, mais larga ou mais chamativa do que o original, mesmo que isso a deixe visualmente mais sutil ou difícil de perceber na imagem gerada.
+Composição: Homem de pele morena clara, cabelo curto penteado para o lado, em pé em um ambiente externo arborizado, uma das mãos no bolso da calça e a outra relaxada ao lado do corpo, expressão descontraída, olhando levemente para baixo. Veste uma camisa de linho bege aberta sobre uma camiseta branca. Luz natural difusa de dia nublado. Enquadramento da cintura para cima, valorizando pulso e mão.
+Fotografia lifestyle hiper-realista para campanha de joias, em formato vertical 3:4 e altíssima resolução. Rosto e expressão da modelo aparecem naturalmente, sem pose rígida ou artificial — a cena deve parecer um flagrante espontâneo do dia a dia, nunca uma fotografia de estúdio posada. Lente equivalente a 85mm, profundidade de campo rasa, fundo suavemente desfocado. A joia permanece perfeitamente nítida e prioritária no foco, com reflexos fisicamente corretos no metal. Pele com textura natural, sem efeito plástico ou de filtro. Mãos, quando aparecerem, devem ter anatomia perfeita — sempre cinco dedos, nunca deformados, duplicados ou fundidos.
+Qualidade: altíssima resolução, nitidez máxima na joia, excelente alcance dinâmico, texturas naturais, reflexos fisicamente corretos, cores absolutamente fiéis, acabamento fotográfico profissional. Eliminar completamente aparência de renderização 3D, ruído digital, granulado, halos ou qualquer aspecto artificial típico de imagem gerada por IA. A peça não deve parecer flutuando, tombada ou fora de escala — preserve rigorosamente suas proporções e comportamento físico real. Antes de finalizar, confirme item por item: a quantidade de peças geradas é idêntica à da foto original (nem a mais, nem a menos); nenhuma peça, pingente ou pedra foi inventado, duplicado ou removido; todos os detalhes de acabamento batem com o original. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr"/>
+      <c r="K11" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:K11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Tipo de Peça</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Pose/Enquadramento</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Tem Modelo?</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Perfis Sugeridos</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Nome de Referência</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Prompt Mestre</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Proporção</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>Link da Imagem Gerada</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>Observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="160" customHeight="1">
+      <c r="A2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Peças em Você</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Retrato Frontal — Colar</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>Sim (requer 2 fotos: sua + joia)</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr"/>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>voce_01_retrato-frontal</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Serão anexadas duas fotografias: a FOTO 1, com o rosto da própria assinante, e a FOTO 2, com a(s) joia(s) do produto. A FOTO 1 determina exclusivamente a identidade da modelo: preserve fielmente formato do rosto, olhos, sobrancelhas, nariz, boca, mandíbula, proporções faciais, tom de pele e cabelo (cor, comprimento e textura reais) — a pessoa da imagem final deve continuar claramente reconhecível como a mesma pessoa da FOTO 1. Não a transforme em um rosto genérico, não rejuvenesça, não altere suas feições ou idade aparente. A FOTO 2 determina exclusivamente as joias: identifique exatamente quantas peças e de que tipo existem nela e utilize somente essas peças, na mesma quantidade — nunca invente, duplique, remova ou substitua nenhuma peça; preserve formato, proporções, espessura, acabamento, brilho, cor do metal, pedras e todos os detalhes originais. Se a FOTO 2 contiver outra pessoa, ignore completamente essa pessoa — rosto, corpo, pele, cabelo, roupa e pose não servem de referência, apenas as joias. Nunca misture as duas fotos: cabelo e tom de pele vêm sempre da FOTO 1; joias vêm sempre da FOTO 2. Se determinado tipo de joia não existir na FOTO 2, ele não deve aparecer na imagem final sob nenhuma hipótese.
+Composição: retrato fechado, mostrando cabeça, pescoço, colo e ombros. O rosto permanece voltado quase totalmente para a câmera, com uma rotação lateral muito sutil e leve inclinação da cabeça para baixo. Olhar direto para a lente, expressão séria e segura, lábios relaxados sem sorriso. Cabelo completamente solto, penteado para trás com efeito levemente úmido, deixando testa, orelhas, pescoço e colo totalmente visíveis. Vestir uma peça preta tomara-que-caia minimalista, ombros e colo à mostra. Fundo liso em cinza-grafite bem escuro. Iluminação de estúdio forte e direcional vinda de um dos lados e ligeiramente de cima: o rosto deve ficar muito iluminado de um lado e com sombra mais marcada do outro, mas pescoço e colo permanecem claros o suficiente para valorizar plenamente o colar. Quando houver brincos, manter as duas orelhas visíveis.
+Qualidade: altíssima resolução, nitidez máxima no rosto e na(s) joia(s), textura de pele natural e realista (sem efeito plástico ou de filtro de beleza), reflexos fisicamente corretos no metal, cores fiéis. Mãos e dedos, quando aparecerem, devem ter anatomia perfeita — sempre cinco dedos, nunca deformados, fundidos ou duplicados, e nunca uma segunda mão ou braço aparecendo acidentalmente no enquadramento. Antes de finalizar, confirme item por item: o rosto ainda é claramente reconhecível como a pessoa da FOTO 1; a quantidade e o tipo de joias são idênticos aos da FOTO 2; nenhuma peça foi inventada, duplicada ou removida. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="inlineStr"/>
+      <c r="K2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3" ht="160" customHeight="1">
+      <c r="A3" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Peças em Você</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Mão no Rosto — Anel e Pulseira</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Sim (requer 2 fotos: sua + joia)</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr"/>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>voce_02_mao-no-rosto</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Serão anexadas duas fotografias: a FOTO 1, com o rosto da própria assinante, e a FOTO 2, com a(s) joia(s) do produto. A FOTO 1 determina exclusivamente a identidade da modelo: preserve fielmente formato do rosto, olhos, sobrancelhas, nariz, boca, mandíbula, proporções faciais, tom de pele e cabelo (cor, comprimento e textura reais) — a pessoa da imagem final deve continuar claramente reconhecível como a mesma pessoa da FOTO 1. Não a transforme em um rosto genérico, não rejuvenesça, não altere suas feições ou idade aparente. A FOTO 2 determina exclusivamente as joias: identifique exatamente quantas peças e de que tipo existem nela e utilize somente essas peças, na mesma quantidade — nunca invente, duplique, remova ou substitua nenhuma peça; preserve formato, proporções, espessura, acabamento, brilho, cor do metal, pedras e todos os detalhes originais. Se a FOTO 2 contiver outra pessoa, ignore completamente essa pessoa — rosto, corpo, pele, cabelo, roupa e pose não servem de referência, apenas as joias. Nunca misture as duas fotos: cabelo e tom de pele vêm sempre da FOTO 1; joias vêm sempre da FOTO 2. Se determinado tipo de joia não existir na FOTO 2, ele não deve aparecer na imagem final sob nenhuma hipótese.
+Composição: retrato fechado do rosto e ombros, com uma das mãos levantada cobrindo parcialmente um dos olhos, dorso da mão voltado para a câmera, dedos estendidos e relaxados. A outra mão não aparece no enquadramento. Expressão neutra e sofisticada, olhar direto para a lente através do espaço entre os dedos. Cabelo solto, repartido ao meio, caindo naturalmente atrás dos ombros. Vestir uma blusa de tricô canelado off-white sem mangas. Fundo liso em bege claro. Iluminação de estúdio suave e lateral, com leve sombra do lado oposto à luz. Quando houver anel, posicioná-lo no dedo correspondente da mão levantada; quando houver pulseira, mantê-la visível no pulso dessa mesma mão.
+Qualidade: altíssima resolução, nitidez máxima no rosto e na(s) joia(s), textura de pele natural e realista (sem efeito plástico ou de filtro de beleza), reflexos fisicamente corretos no metal, cores fiéis. Mãos e dedos, quando aparecerem, devem ter anatomia perfeita — sempre cinco dedos, nunca deformados, fundidos ou duplicados, e nunca uma segunda mão ou braço aparecendo acidentalmente no enquadramento. Antes de finalizar, confirme item por item: o rosto ainda é claramente reconhecível como a pessoa da FOTO 1; a quantidade e o tipo de joias são idênticos aos da FOTO 2; nenhuma peça foi inventada, duplicada ou removida. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr"/>
+      <c r="K3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4" ht="160" customHeight="1">
+      <c r="A4" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Peças em Você</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Perfil com Coque — Brinco e Colar</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Sim (requer 2 fotos: sua + joia)</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr"/>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>voce_03_perfil-com-coque</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Serão anexadas duas fotografias: a FOTO 1, com o rosto da própria assinante, e a FOTO 2, com a(s) joia(s) do produto. A FOTO 1 determina exclusivamente a identidade da modelo: preserve fielmente formato do rosto, olhos, sobrancelhas, nariz, boca, mandíbula, proporções faciais, tom de pele e cabelo (cor, comprimento e textura reais) — a pessoa da imagem final deve continuar claramente reconhecível como a mesma pessoa da FOTO 1. Não a transforme em um rosto genérico, não rejuvenesça, não altere suas feições ou idade aparente. A FOTO 2 determina exclusivamente as joias: identifique exatamente quantas peças e de que tipo existem nela e utilize somente essas peças, na mesma quantidade — nunca invente, duplique, remova ou substitua nenhuma peça; preserve formato, proporções, espessura, acabamento, brilho, cor do metal, pedras e todos os detalhes originais. Se a FOTO 2 contiver outra pessoa, ignore completamente essa pessoa — rosto, corpo, pele, cabelo, roupa e pose não servem de referência, apenas as joias. Nunca misture as duas fotos: cabelo e tom de pele vêm sempre da FOTO 1; joias vêm sempre da FOTO 2. Se determinado tipo de joia não existir na FOTO 2, ele não deve aparecer na imagem final sob nenhuma hipótese.
+Composição: retrato fechado em perfil de aproximadamente três quartos, cabeça claramente virada para o lado, queixo levemente elevado, pescoço alongado e visível. Olhar direcionado para o lado, fora do enquadramento. Lábios levemente entreabertos, sem sorriso. Cabelo preso em coque alto, deixando nuca, pescoço e orelha completamente visíveis. Vestir uma camisa branca ampla, caída sobre os ombros, decote em V comportado, sem expor o colo além das clavículas. Fundo liso em tom terracota quente. Iluminação de estúdio lateral e suave, destacando claramente pescoço, orelha e colo. Quando houver colar, mantê-lo totalmente visível sobre o colo; quando houver brinco, a orelha do lado virado para a câmera permanece livre de cabelo.
+Qualidade: altíssima resolução, nitidez máxima no rosto e na(s) joia(s), textura de pele natural e realista (sem efeito plástico ou de filtro de beleza), reflexos fisicamente corretos no metal, cores fiéis. Mãos e dedos, quando aparecerem, devem ter anatomia perfeita — sempre cinco dedos, nunca deformados, fundidos ou duplicados, e nunca uma segunda mão ou braço aparecendo acidentalmente no enquadramento. Antes de finalizar, confirme item por item: o rosto ainda é claramente reconhecível como a pessoa da FOTO 1; a quantidade e o tipo de joias são idênticos aos da FOTO 2; nenhuma peça foi inventada, duplicada ou removida. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr"/>
+      <c r="K4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5" ht="160" customHeight="1">
+      <c r="A5" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Peças em Você</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Mão na Cabeça — Anel</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Sim (requer 2 fotos: sua + joia)</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr"/>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>voce_04_mao-na-cabeca</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Serão anexadas duas fotografias: a FOTO 1, com o rosto da própria assinante, e a FOTO 2, com a(s) joia(s) do produto. A FOTO 1 determina exclusivamente a identidade da modelo: preserve fielmente formato do rosto, olhos, sobrancelhas, nariz, boca, mandíbula, proporções faciais, tom de pele e cabelo (cor, comprimento e textura reais) — a pessoa da imagem final deve continuar claramente reconhecível como a mesma pessoa da FOTO 1. Não a transforme em um rosto genérico, não rejuvenesça, não altere suas feições ou idade aparente. A FOTO 2 determina exclusivamente as joias: identifique exatamente quantas peças e de que tipo existem nela e utilize somente essas peças, na mesma quantidade — nunca invente, duplique, remova ou substitua nenhuma peça; preserve formato, proporções, espessura, acabamento, brilho, cor do metal, pedras e todos os detalhes originais. Se a FOTO 2 contiver outra pessoa, ignore completamente essa pessoa — rosto, corpo, pele, cabelo, roupa e pose não servem de referência, apenas as joias. Nunca misture as duas fotos: cabelo e tom de pele vêm sempre da FOTO 1; joias vêm sempre da FOTO 2. Se determinado tipo de joia não existir na FOTO 2, ele não deve aparecer na imagem final sob nenhuma hipótese.
+Composição: retrato fechado em perfil de três quartos, um dos braços dobrado para cima com a mão apoiada delicadamente na lateral da cabeça, próxima à têmpora — os dedos tocam apenas o cabelo, sem pressionar o rosto. Cotovelo apoiado sobre uma superfície fora de quadro. A outra mão não aparece. Olhar direcionado para o lado, expressão tranquila. Cabelo solto caindo sobre o ombro oposto ao braço levantado. Vestir uma blusa preta simples de alças finas. Fundo liso em cinza claro. Iluminação suave e difusa, levemente lateral. Quando houver anel, posicioná-lo no dedo visível da mão levantada.
+Qualidade: altíssima resolução, nitidez máxima no rosto e na(s) joia(s), textura de pele natural e realista (sem efeito plástico ou de filtro de beleza), reflexos fisicamente corretos no metal, cores fiéis. Mãos e dedos, quando aparecerem, devem ter anatomia perfeita — sempre cinco dedos, nunca deformados, fundidos ou duplicados, e nunca uma segunda mão ou braço aparecendo acidentalmente no enquadramento. Antes de finalizar, confirme item por item: o rosto ainda é claramente reconhecível como a pessoa da FOTO 1; a quantidade e o tipo de joias são idênticos aos da FOTO 2; nenhuma peça foi inventada, duplicada ou removida. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr"/>
+      <c r="K5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6" ht="160" customHeight="1">
+      <c r="A6" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Peças em Você</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Cadeira ao Contrário — Conjunto</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Sim (requer 2 fotos: sua + joia)</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr"/>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>voce_05_cadeira-ao-contrario</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Serão anexadas duas fotografias: a FOTO 1, com o rosto da própria assinante, e a FOTO 2, com a(s) joia(s) do produto. A FOTO 1 determina exclusivamente a identidade da modelo: preserve fielmente formato do rosto, olhos, sobrancelhas, nariz, boca, mandíbula, proporções faciais, tom de pele e cabelo (cor, comprimento e textura reais) — a pessoa da imagem final deve continuar claramente reconhecível como a mesma pessoa da FOTO 1. Não a transforme em um rosto genérico, não rejuvenesça, não altere suas feições ou idade aparente. A FOTO 2 determina exclusivamente as joias: identifique exatamente quantas peças e de que tipo existem nela e utilize somente essas peças, na mesma quantidade — nunca invente, duplique, remova ou substitua nenhuma peça; preserve formato, proporções, espessura, acabamento, brilho, cor do metal, pedras e todos os detalhes originais. Se a FOTO 2 contiver outra pessoa, ignore completamente essa pessoa — rosto, corpo, pele, cabelo, roupa e pose não servem de referência, apenas as joias. Nunca misture as duas fotos: cabelo e tom de pele vêm sempre da FOTO 1; joias vêm sempre da FOTO 2. Se determinado tipo de joia não existir na FOTO 2, ele não deve aparecer na imagem final sob nenhuma hipótese.
+Composição: modelo sentada ao contrário em uma cadeira branca minimalista, encosto voltado para a frente do corpo, tronco e cadeira levemente girados em diagonal (cerca de 20 a 30 graus) em relação à câmera. Um braço cruza a frente do encosto; o outro sobe com o cotovelo apoiado sobre o encosto e a mão repousando perto da têmpora. Cabeça inclinada suavemente em direção a essa mão, olhos voltados para a câmera, expressão tranquila e lábios levemente entreabertos. Cabelo preso em coque baixo com fios soltos ao redor do rosto. Vestir uma regata preta simples. Fundo liso off-white. Iluminação difusa e lateral, acompanhando a diagonal da pose. Quando houver pulseira, ela deve ficar no pulso da mão próxima ao rosto; quando houver colar e brincos, ambos permanecem visíveis e bem iluminados.
+Qualidade: altíssima resolução, nitidez máxima no rosto e na(s) joia(s), textura de pele natural e realista (sem efeito plástico ou de filtro de beleza), reflexos fisicamente corretos no metal, cores fiéis. Mãos e dedos, quando aparecerem, devem ter anatomia perfeita — sempre cinco dedos, nunca deformados, fundidos ou duplicados, e nunca uma segunda mão ou braço aparecendo acidentalmente no enquadramento. Antes de finalizar, confirme item por item: o rosto ainda é claramente reconhecível como a pessoa da FOTO 1; a quantidade e o tipo de joias são idênticos aos da FOTO 2; nenhuma peça foi inventada, duplicada ou removida. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr"/>
+      <c r="K6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7" ht="160" customHeight="1">
+      <c r="A7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Peças em Você</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Debruçada na Mesa — Colar e Brinco</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Sim (requer 2 fotos: sua + joia)</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr"/>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>voce_06_debrucada-na-mesa</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Serão anexadas duas fotografias: a FOTO 1, com o rosto da própria assinante, e a FOTO 2, com a(s) joia(s) do produto. A FOTO 1 determina exclusivamente a identidade da modelo: preserve fielmente formato do rosto, olhos, sobrancelhas, nariz, boca, mandíbula, proporções faciais, tom de pele e cabelo (cor, comprimento e textura reais) — a pessoa da imagem final deve continuar claramente reconhecível como a mesma pessoa da FOTO 1. Não a transforme em um rosto genérico, não rejuvenesça, não altere suas feições ou idade aparente. A FOTO 2 determina exclusivamente as joias: identifique exatamente quantas peças e de que tipo existem nela e utilize somente essas peças, na mesma quantidade — nunca invente, duplique, remova ou substitua nenhuma peça; preserve formato, proporções, espessura, acabamento, brilho, cor do metal, pedras e todos os detalhes originais. Se a FOTO 2 contiver outra pessoa, ignore completamente essa pessoa — rosto, corpo, pele, cabelo, roupa e pose não servem de referência, apenas as joias. Nunca misture as duas fotos: cabelo e tom de pele vêm sempre da FOTO 1; joias vêm sempre da FOTO 2. Se determinado tipo de joia não existir na FOTO 2, ele não deve aparecer na imagem final sob nenhuma hipótese.
+Composição: modelo debruçada sobre uma mesa branca lisa, tronco inclinado para frente e levemente para o lado, um ombro mais próximo da câmera que o outro. Um braço sobe com a mão apoiada na lateral superior da cabeça, sobre o cabelo, sem cobrir a testa; o outro braço fica totalmente apoiado sobre a mesa, mão relaxada sobre a superfície, sem tocar o outro braço. Olhar direto para a câmera, expressão segura e elegante, sem sinais de cansaço. Cabelo solto, penteado para trás. Vestir uma camisa branca ampla e moderna. Fundo liso em cinza claro. Iluminação de estúdio clara e lateral, com sombras suaves da mesa e dos braços. Quando houver colar, mantê-lo visível sobre o colo; quando houver brinco, a orelha correspondente permanece livre; quando houver anel, posicioná-lo na mão apoiada sobre a mesa.
+Qualidade: altíssima resolução, nitidez máxima no rosto e na(s) joia(s), textura de pele natural e realista (sem efeito plástico ou de filtro de beleza), reflexos fisicamente corretos no metal, cores fiéis. Mãos e dedos, quando aparecerem, devem ter anatomia perfeita — sempre cinco dedos, nunca deformados, fundidos ou duplicados, e nunca uma segunda mão ou braço aparecendo acidentalmente no enquadramento. Antes de finalizar, confirme item por item: o rosto ainda é claramente reconhecível como a pessoa da FOTO 1; a quantidade e o tipo de joias são idênticos aos da FOTO 2; nenhuma peça foi inventada, duplicada ou removida. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr"/>
+      <c r="K7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8" ht="160" customHeight="1">
+      <c r="A8" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Peças em Você</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Regata Frontal — Colar</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Sim (requer 2 fotos: sua + joia)</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr"/>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>voce_07_regata-frontal</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Serão anexadas duas fotografias: a FOTO 1, com o rosto da própria assinante, e a FOTO 2, com a(s) joia(s) do produto. A FOTO 1 determina exclusivamente a identidade da modelo: preserve fielmente formato do rosto, olhos, sobrancelhas, nariz, boca, mandíbula, proporções faciais, tom de pele e cabelo (cor, comprimento e textura reais) — a pessoa da imagem final deve continuar claramente reconhecível como a mesma pessoa da FOTO 1. Não a transforme em um rosto genérico, não rejuvenesça, não altere suas feições ou idade aparente. A FOTO 2 determina exclusivamente as joias: identifique exatamente quantas peças e de que tipo existem nela e utilize somente essas peças, na mesma quantidade — nunca invente, duplique, remova ou substitua nenhuma peça; preserve formato, proporções, espessura, acabamento, brilho, cor do metal, pedras e todos os detalhes originais. Se a FOTO 2 contiver outra pessoa, ignore completamente essa pessoa — rosto, corpo, pele, cabelo, roupa e pose não servem de referência, apenas as joias. Nunca misture as duas fotos: cabelo e tom de pele vêm sempre da FOTO 1; joias vêm sempre da FOTO 2. Se determinado tipo de joia não existir na FOTO 2, ele não deve aparecer na imagem final sob nenhuma hipótese.
+Composição: retrato fechado quase frontal, corpo levemente apoiado contra uma parede lisa atrás, ombros relaxados, cabeça praticamente reta com inclinação mínima. Olhar direto para a câmera, expressão neutra e contemporânea, lábios relaxados e suavemente entreabertos. Cabelo solto com leve movimento, uma mecha podendo cruzar parte do rosto de forma natural, mantendo pelo menos um olho sempre visível. Vestir uma regata preta lisa e minimalista, decote arredondado moderado. Fundo em parede branca lisa. Iluminação natural lateral, criando sombra suave da modelo sobre a parede ao fundo. Quando houver colar, o decote deve deixá-lo totalmente visível sobre o colo.
+Qualidade: altíssima resolução, nitidez máxima no rosto e na(s) joia(s), textura de pele natural e realista (sem efeito plástico ou de filtro de beleza), reflexos fisicamente corretos no metal, cores fiéis. Mãos e dedos, quando aparecerem, devem ter anatomia perfeita — sempre cinco dedos, nunca deformados, fundidos ou duplicados, e nunca uma segunda mão ou braço aparecendo acidentalmente no enquadramento. Antes de finalizar, confirme item por item: o rosto ainda é claramente reconhecível como a pessoa da FOTO 1; a quantidade e o tipo de joias são idênticos aos da FOTO 2; nenhuma peça foi inventada, duplicada ou removida. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr"/>
+      <c r="K8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9" ht="160" customHeight="1">
+      <c r="A9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Peças em Você</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Vento no Cabelo — Brinco</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Sim (requer 2 fotos: sua + joia)</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr"/>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>voce_08_vento-no-cabelo</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Serão anexadas duas fotografias: a FOTO 1, com o rosto da própria assinante, e a FOTO 2, com a(s) joia(s) do produto. A FOTO 1 determina exclusivamente a identidade da modelo: preserve fielmente formato do rosto, olhos, sobrancelhas, nariz, boca, mandíbula, proporções faciais, tom de pele e cabelo (cor, comprimento e textura reais) — a pessoa da imagem final deve continuar claramente reconhecível como a mesma pessoa da FOTO 1. Não a transforme em um rosto genérico, não rejuvenesça, não altere suas feições ou idade aparente. A FOTO 2 determina exclusivamente as joias: identifique exatamente quantas peças e de que tipo existem nela e utilize somente essas peças, na mesma quantidade — nunca invente, duplique, remova ou substitua nenhuma peça; preserve formato, proporções, espessura, acabamento, brilho, cor do metal, pedras e todos os detalhes originais. Se a FOTO 2 contiver outra pessoa, ignore completamente essa pessoa — rosto, corpo, pele, cabelo, roupa e pose não servem de referência, apenas as joias. Nunca misture as duas fotos: cabelo e tom de pele vêm sempre da FOTO 1; joias vêm sempre da FOTO 2. Se determinado tipo de joia não existir na FOTO 2, ele não deve aparecer na imagem final sob nenhuma hipótese.
+Composição: retrato fechado frontal, corpo praticamente reto e relaxado, cabeça reta, olhar direto para a câmera. O cabelo aparece solto e movimentado lateralmente por vento, com uma mecha cruzando parte do rosto e um dos olhos, mantendo a outra metade do rosto e uma orelha completamente visíveis. Expressão tranquila e natural. Vestir uma camisa social clara aberta nos ombros. Fundo liso e neutro. Iluminação lateral suave, simulando luz de sol filtrada. Quando houver brinco, a orelha visível deve ficar totalmente livre de cabelo para destacá-lo.
+Qualidade: altíssima resolução, nitidez máxima no rosto e na(s) joia(s), textura de pele natural e realista (sem efeito plástico ou de filtro de beleza), reflexos fisicamente corretos no metal, cores fiéis. Mãos e dedos, quando aparecerem, devem ter anatomia perfeita — sempre cinco dedos, nunca deformados, fundidos ou duplicados, e nunca uma segunda mão ou braço aparecendo acidentalmente no enquadramento. Antes de finalizar, confirme item por item: o rosto ainda é claramente reconhecível como a pessoa da FOTO 1; a quantidade e o tipo de joias são idênticos aos da FOTO 2; nenhuma peça foi inventada, duplicada ou removida. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="inlineStr"/>
+      <c r="K9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10" ht="160" customHeight="1">
+      <c r="A10" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Peças em Você</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Apoiada em Cadeira — Pulseira</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Sim (requer 2 fotos: sua + joia)</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr"/>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>voce_09_apoiada-em-cadeira</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Serão anexadas duas fotografias: a FOTO 1, com o rosto da própria assinante, e a FOTO 2, com a(s) joia(s) do produto. A FOTO 1 determina exclusivamente a identidade da modelo: preserve fielmente formato do rosto, olhos, sobrancelhas, nariz, boca, mandíbula, proporções faciais, tom de pele e cabelo (cor, comprimento e textura reais) — a pessoa da imagem final deve continuar claramente reconhecível como a mesma pessoa da FOTO 1. Não a transforme em um rosto genérico, não rejuvenesça, não altere suas feições ou idade aparente. A FOTO 2 determina exclusivamente as joias: identifique exatamente quantas peças e de que tipo existem nela e utilize somente essas peças, na mesma quantidade — nunca invente, duplique, remova ou substitua nenhuma peça; preserve formato, proporções, espessura, acabamento, brilho, cor do metal, pedras e todos os detalhes originais. Se a FOTO 2 contiver outra pessoa, ignore completamente essa pessoa — rosto, corpo, pele, cabelo, roupa e pose não servem de referência, apenas as joias. Nunca misture as duas fotos: cabelo e tom de pele vêm sempre da FOTO 1; joias vêm sempre da FOTO 2. Se determinado tipo de joia não existir na FOTO 2, ele não deve aparecer na imagem final sob nenhuma hipótese.
+Composição: modelo em pé, apoiada casualmente no encosto de uma cadeira branca minimalista, um braço apoiado sobre o encosto com o pulso e a mão relaxados e visíveis, o outro braço relaxado ao lado do corpo. Corpo levemente girado em relação à câmera, olhar direto para a lente, expressão serena. Cabelo solto com ondas suaves. Vestir uma camisa de linho bege. Fundo liso em tom areia. Iluminação suave e natural, lateral. Quando houver pulseira, ela deve ficar visível no pulso apoiado sobre o encosto da cadeira.
+Qualidade: altíssima resolução, nitidez máxima no rosto e na(s) joia(s), textura de pele natural e realista (sem efeito plástico ou de filtro de beleza), reflexos fisicamente corretos no metal, cores fiéis. Mãos e dedos, quando aparecerem, devem ter anatomia perfeita — sempre cinco dedos, nunca deformados, fundidos ou duplicados, e nunca uma segunda mão ou braço aparecendo acidentalmente no enquadramento. Antes de finalizar, confirme item por item: o rosto ainda é claramente reconhecível como a pessoa da FOTO 1; a quantidade e o tipo de joias são idênticos aos da FOTO 2; nenhuma peça foi inventada, duplicada ou removida. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr"/>
+      <c r="K10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11" ht="160" customHeight="1">
+      <c r="A11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Peças em Você</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Espelho com Celular — Brinco</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Sim (requer 2 fotos: sua + joia)</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr"/>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>voce_10_espelho-com-celular</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Serão anexadas duas fotografias: a FOTO 1, com o rosto da própria assinante, e a FOTO 2, com a(s) joia(s) do produto. A FOTO 1 determina exclusivamente a identidade da modelo: preserve fielmente formato do rosto, olhos, sobrancelhas, nariz, boca, mandíbula, proporções faciais, tom de pele e cabelo (cor, comprimento e textura reais) — a pessoa da imagem final deve continuar claramente reconhecível como a mesma pessoa da FOTO 1. Não a transforme em um rosto genérico, não rejuvenesça, não altere suas feições ou idade aparente. A FOTO 2 determina exclusivamente as joias: identifique exatamente quantas peças e de que tipo existem nela e utilize somente essas peças, na mesma quantidade — nunca invente, duplique, remova ou substitua nenhuma peça; preserve formato, proporções, espessura, acabamento, brilho, cor do metal, pedras e todos os detalhes originais. Se a FOTO 2 contiver outra pessoa, ignore completamente essa pessoa — rosto, corpo, pele, cabelo, roupa e pose não servem de referência, apenas as joias. Nunca misture as duas fotos: cabelo e tom de pele vêm sempre da FOTO 1; joias vêm sempre da FOTO 2. Se determinado tipo de joia não existir na FOTO 2, ele não deve aparecer na imagem final sob nenhuma hipótese.
+Composição: modelo em pé diante de um espelho de moldura fina preta com cantos arredondados, segurando um smartphone com as duas mãos em frente ao rosto, cobrindo boa parte dele — apenas testa, cabelo, mandíbula e uma orelha permanecem visíveis. Cabelo solto, penteado atrás da orelha visível. Vestir uma camisa branca oversized com um ombro levemente à mostra. Fundo minimalista, parede lisa em cinza muito claro. Iluminação suave, sugerindo uma janela fora do enquadramento, incidindo lateralmente. Quando houver brinco, a orelha visível deve permanecer totalmente livre de cabelo para destacá-lo.
+Qualidade: altíssima resolução, nitidez máxima no rosto e na(s) joia(s), textura de pele natural e realista (sem efeito plástico ou de filtro de beleza), reflexos fisicamente corretos no metal, cores fiéis. Mãos e dedos, quando aparecerem, devem ter anatomia perfeita — sempre cinco dedos, nunca deformados, fundidos ou duplicados, e nunca uma segunda mão ou braço aparecendo acidentalmente no enquadramento. Antes de finalizar, confirme item por item: o rosto ainda é claramente reconhecível como a pessoa da FOTO 1; a quantidade e o tipo de joias são idênticos aos da FOTO 2; nenhuma peça foi inventada, duplicada ou removida. Formato final da imagem: 3:4 (vertical).</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>3:4 (vertical)</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>A gerar</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr"/>
+      <c r="K11" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:K11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>